<commit_message>
Integrate real Kalodata data into Toni Black strategy
- Add real top-15 products (Men's Underwear ID, 30d) confirming Rp100rb tier
  is dominated by 3-6pcs bundles (~Rp15-33rb/pcs) — validates Toni Black's
  single-pcs premium white space
- Add top-10 creators/affiliates + winning video formats from Kalodata
- Revise strategy: micro-influencer affiliate engine, mandatory live
  shopping, paid/Spark Ads layer, market-saturation red flag
- Two new workbook sheets: Kalodata Top Produk, Creator & Format

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FdFYs9Ji5gfr8VFihGLxdU
</commit_message>
<xml_diff>
--- a/toni-black/toni-black-content-planning.xlsx
+++ b/toni-black/toni-black-content-planning.xlsx
@@ -10,9 +10,11 @@
     <sheet name="Panduan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Content Pillars" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Riset Kompetitor" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hook Bank" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Planning 30 Hari" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Performance Tracker" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Kalodata - Top Produk" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Kalodata - Creator &amp; Format" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hook Bank" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Planning 30 Hari" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Performance Tracker" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,12 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD MMM YYYY"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="DD MMM YYYY"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +70,14 @@
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -122,6 +129,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00595959"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -149,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,7 +204,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -213,7 +225,7 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -222,19 +234,37 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1258,6 +1288,1205 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Produk (ringkas)</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Toko / Brand</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Harga 'Paket'</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Isi Paket</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Est. Harga/pcs</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Terjual (30 hr)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Revenue (30 hr)</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Positioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Boxer olahraga anti-wear, cepat kering</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>uncolive.underwear</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Rp102.447</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs (beli 4 gratis 2)</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>± Rp17rb</t>
+        </is>
+      </c>
+      <c r="G2" s="39" t="n">
+        <v>14450</v>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Rp1,48 M</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Sports, quick-dry, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Sports underwear 'French' marathon</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>uomolive</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Rp91.387</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs (beli 4 gratis 2)</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>± Rp15rb</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="n">
+        <v>10498</v>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Rp959 jt</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Sports, seamless, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>S9002 sports underwear anti-wear</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>uomolive</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Rp118.743</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs (beli 4 gratis 2)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>± Rp20rb</t>
+        </is>
+      </c>
+      <c r="G4" s="39" t="n">
+        <v>6201</v>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Rp736 jt</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Sports, quick-dry, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Ryusei Boxer Haruki</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Ryusei</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Rp95.036</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>3 pcs</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>± Rp32rb</t>
+        </is>
+      </c>
+      <c r="G5" s="39" t="n">
+        <v>5682</v>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Rp540 jt</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Nyaman &amp; elastis, brand lokal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Boxer Premium Anti Bakteri</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Vallero Store</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Rp101.661</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>± Rp17rb</t>
+        </is>
+      </c>
+      <c r="G6" s="39" t="n">
+        <v>5029</v>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Rp511 jt</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Antibakteri, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Boxer Ice Silk antibakteri</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Michiyo</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Rp93.883</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>± Rp16rb</t>
+        </is>
+      </c>
+      <c r="G7" s="39" t="n">
+        <v>4331</v>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Rp407 jt</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Ice silk, seamless, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>VAUDREÉ paket hemat Ice Silk</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>VAUDREE</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Rp82.415</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>4 pcs</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>± Rp21rb</t>
+        </is>
+      </c>
+      <c r="G8" s="39" t="n">
+        <v>4266</v>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Rp352 jt</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Ice silk premium, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>JFYOU katun premium (buy 1 get 3)</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>SUANKA STORE</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Rp88.319</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>4 pcs</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>± Rp22rb</t>
+        </is>
+      </c>
+      <c r="G9" s="39" t="n">
+        <v>3188</v>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Rp282 jt</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Katun premium, viral, COD</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Crossbell x Moow Ice Silk 7A</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Crossbell Store</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Rp123.291</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>4 pcs</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>± Rp31rb</t>
+        </is>
+      </c>
+      <c r="G10" s="39" t="n">
+        <v>1886</v>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Rp233 jt</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Ice silk premium, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Combo boxer poly polos</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>LEADER.CO</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Rp90.958</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>± Rp15rb</t>
+        </is>
+      </c>
+      <c r="G11" s="39" t="n">
+        <v>2088</v>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Rp190 jt</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Basic polos, uniseks, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>VIMISU Boxer seamless antibakteri</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>VIMISU 1</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Rp86.555</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>varian (L-5XL)</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="39" t="n">
+        <v>1992</v>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Rp172 jt</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Seamless, antibakteri, motif</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>HEPNIES boxer teknologi magnet</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>HEPNIES MEN'S UNDERWEAR</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Rp97.527</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>3 pcs</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>± Rp33rb</t>
+        </is>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>1728</v>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Rp169 jt</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Gimmick teknologi, ringan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>9003 celana lari Prancis anti-wear</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>uomolive</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Rp121.687</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs (beli 4 gratis 2)</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>± Rp20rb</t>
+        </is>
+      </c>
+      <c r="G14" s="39" t="n">
+        <v>1106</v>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Rp135 jt</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Sports, quick-dry, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Boxer Ice Silk paket hemat</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Starwing</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Rp117.712</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>± Rp20rb</t>
+        </is>
+      </c>
+      <c r="G15" s="39" t="n">
+        <v>1083</v>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Rp127 jt</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Ice silk, antibakteri, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>VAUDREÉ paket hemat Ice Silk</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>VAUDREE</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Rp109.370</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>6 pcs (L-6XL)</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>± Rp18rb</t>
+        </is>
+      </c>
+      <c r="G16" s="39" t="n">
+        <v>1117</v>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Rp122 jt</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Ice silk premium, bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>INSIGHT: Semua produk teratas di tier Rp80–150rb adalah BUNDLE 3–6 pcs → harga efektif hanya ± Rp15–33rb/pcs. Tidak ada satu pun produk 1 pcs premium seharga Rp100rb di ranking. Toni Black (Rp100rb/1 pcs premium) praktis tanpa kompetitor langsung — tantangannya edukasi persepsi harga, bukan mengalahkan brand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="inlineStr">
+        <is>
+          <t>Sumber: Kalodata (KaloPilot), kategori Men's Underwear ID 841352, region ID, 30 hari terakhir, ditarik 20 Juli 2026. 'Est. harga/pcs' = harga paket dibagi jumlah isi (perkiraan).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A19:I19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="40" t="inlineStr">
+        <is>
+          <t>TOP CREATOR / AFFILIATE (revenue tertinggi, 30 hari)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="41" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="41" t="inlineStr">
+        <is>
+          <t>Creator (handle)</t>
+        </is>
+      </c>
+      <c r="C2" s="41" t="inlineStr">
+        <is>
+          <t>Follower</t>
+        </is>
+      </c>
+      <c r="D2" s="41" t="inlineStr">
+        <is>
+          <t>Revenue (30 hr)</t>
+        </is>
+      </c>
+      <c r="E2" s="41" t="inlineStr">
+        <is>
+          <t>Model &amp; Catatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>JURAGAN SEMPAK (@user835006894)</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="n">
+        <v>3402</v>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Rp452 jt</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>100% video. Micro-follower tapi revenue #1 → targeting tajam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Ryan Outfitness (@ryan.outfitness)</t>
+        </is>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>9574</v>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Rp439 jt</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid: 98% revenue dari LIVE, video jadi funnel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Ko.ony (@ko.ony96)</t>
+        </is>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>65700</v>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Rp411 jt</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Fokus video, follower besar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>JRshop88 (@jrshop_08)</t>
+        </is>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>17200</v>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Rp361 jt</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid (mayoritas live).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>CK Underwear Store (@ck_underwear_store)</t>
+        </is>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>5153</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Rp339 jt</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>100% LIVE, AOV ~Rp356rb/item (tertinggi!) → segmen mau bayar mahal saat di-edukasi live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>rumahcivi (@rumahcivi)</t>
+        </is>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>92200</v>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Rp329 jt</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Video, follower besar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Promo harian (@promoharian12)</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>1482</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Rp322 jt</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Video AI, follower terkecil, volume tertinggi (5.715 sales).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>BANG RAB (@bang.rab22)</t>
+        </is>
+      </c>
+      <c r="C10" s="39" t="n">
+        <v>48400</v>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Rp312 jt</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Video, volume sales tertinggi (13.267).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Spesialis Underwear (@spill_underwear)</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="n">
+        <v>2683</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Rp310 jt</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid (mayoritas live), micro-follower.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>sulastridua2 (@sulastridua2)</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="n">
+        <v>44000</v>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Rp306 jt</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid, GROWTH +283% → bintang naik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>FORMAT VIDEO YANG MENANG (analisis 50 video teratas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>Durasi</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>GPM (per 1000 views)</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>Ciri Khas</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Short-form promo</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>5–20 detik</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Rp33rb–763rb</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Produk langsung di 3 detik pertama, hashtag agresif (#cdpria #boxerpria #fyp), fokus visual + promo, no intro.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Demo + bundle detail</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>60–80 detik</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>s/d Rp86rb (tertinggi konsisten)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Tunjuk bahan (katun/ice silk/seamless), close-up/slow-mo tekstur, angle berbagai sisi, bundle promo.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Testimoni + unboxing</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>15–30 detik</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Rp60rb–80rb</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Unboxing excited, review singkat (lembut/adem/nyaman), size chart &amp; pilihan warna, CTA keranjang kuning.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Ultra-short AI video</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>5–10 detik</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>s/d Rp763rb (INSANE)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>AI-generated, hampir 100% dari paid ads, pure product showcase tanpa narasi, biaya produksi rendah.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>IMPLIKASI UNTUK TONI BLACK:</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>1. 98% video top-revenue = PAID ADS. Skala butuh budget iklan (Spark Ads), tapi menang di kualitas kreatif &amp; brand — bukan perang harga (kompetitor bundle sedang jenuh, growth -5% s/d -50%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2. Micro-influencer 1.500–5.000 follower menghasilkan Rp300–450 jt. Bangun program AFFILIATE/seeding ke micro-creator niche (grooming pria, couple/istri) + sediakan sample, script, komisi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>3. LIVE SHOPPING wajib — ~50% revenue kategori dari live; CK Underwear 100% live dengan AOV Rp356rb membuktikan segmen mau bayar premium saat di-edukasi live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>4. Pillar 2 (Tes &amp; Demo) Toni Black = format demo 60–80 detik yang terbukti GPM tinggi. Perkuat itu sebagai materi Spark Ads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>Sumber: Kalodata (KaloPilot), kategori Men's Underwear ID 841352, region ID, 30 hari terakhir, ditarik 20 Juli 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A27:E27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1492,7 +2721,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1584,7 +2813,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="n">
+      <c r="A2" s="42" t="n">
         <v>46230</v>
       </c>
       <c r="B2" s="10" t="inlineStr">
@@ -1645,7 +2874,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="n">
+      <c r="A3" s="42" t="n">
         <v>46231</v>
       </c>
       <c r="B3" s="10" t="inlineStr">
@@ -1706,7 +2935,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="n">
+      <c r="A4" s="42" t="n">
         <v>46232</v>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -1767,7 +2996,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="n">
+      <c r="A5" s="42" t="n">
         <v>46233</v>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -1828,7 +3057,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n">
+      <c r="A6" s="42" t="n">
         <v>46234</v>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -1889,7 +3118,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="n">
+      <c r="A7" s="42" t="n">
         <v>46235</v>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -1950,7 +3179,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n">
+      <c r="A8" s="42" t="n">
         <v>46236</v>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -2011,7 +3240,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="n">
+      <c r="A9" s="42" t="n">
         <v>46237</v>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -2072,7 +3301,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n">
+      <c r="A10" s="42" t="n">
         <v>46238</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -2133,7 +3362,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="n">
+      <c r="A11" s="42" t="n">
         <v>46239</v>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -2194,7 +3423,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n">
+      <c r="A12" s="42" t="n">
         <v>46240</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -2255,7 +3484,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="n">
+      <c r="A13" s="42" t="n">
         <v>46241</v>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -2316,7 +3545,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="42" t="n">
         <v>46242</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -2377,7 +3606,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="n">
+      <c r="A15" s="42" t="n">
         <v>46243</v>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -2438,7 +3667,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="A16" s="42" t="n">
         <v>46244</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -2499,7 +3728,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="n">
+      <c r="A17" s="42" t="n">
         <v>46245</v>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -2560,7 +3789,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="n">
+      <c r="A18" s="42" t="n">
         <v>46246</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -2621,7 +3850,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="n">
+      <c r="A19" s="42" t="n">
         <v>46247</v>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -2682,7 +3911,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n">
+      <c r="A20" s="42" t="n">
         <v>46248</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -2743,7 +3972,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="n">
+      <c r="A21" s="42" t="n">
         <v>46249</v>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -2804,7 +4033,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="n">
+      <c r="A22" s="42" t="n">
         <v>46250</v>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -2865,7 +4094,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="n">
+      <c r="A23" s="42" t="n">
         <v>46251</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -2926,7 +4155,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="n">
+      <c r="A24" s="42" t="n">
         <v>46252</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -2987,7 +4216,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="n">
+      <c r="A25" s="42" t="n">
         <v>46253</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -3048,7 +4277,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="n">
+      <c r="A26" s="42" t="n">
         <v>46254</v>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -3109,7 +4338,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="n">
+      <c r="A27" s="42" t="n">
         <v>46255</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -3170,7 +4399,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="n">
+      <c r="A28" s="42" t="n">
         <v>46256</v>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -3231,7 +4460,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="n">
+      <c r="A29" s="42" t="n">
         <v>46257</v>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -3292,7 +4521,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="n">
+      <c r="A30" s="42" t="n">
         <v>46258</v>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -3353,7 +4582,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="n">
+      <c r="A31" s="42" t="n">
         <v>46259</v>
       </c>
       <c r="B31" s="10" t="inlineStr">
@@ -3418,7 +4647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3516,7 +4745,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="n">
+      <c r="A2" s="43" t="n">
         <v>46230</v>
       </c>
       <c r="B2" s="26" t="inlineStr">
@@ -3558,7 +4787,7 @@
       <c r="L2" s="27" t="n">
         <v>1250000</v>
       </c>
-      <c r="M2" s="28">
+      <c r="M2" s="44">
         <f>IF(OR(E2="",E2=0),"",(F2+G2+H2+I2)/E2)</f>
         <v/>
       </c>
@@ -3568,7 +4797,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n"/>
+      <c r="A3" s="45" t="n"/>
       <c r="B3" s="31" t="n"/>
       <c r="C3" s="31" t="n"/>
       <c r="D3" s="31" t="n"/>
@@ -3580,7 +4809,7 @@
       <c r="J3" s="31" t="n"/>
       <c r="K3" s="31" t="n"/>
       <c r="L3" s="32" t="n"/>
-      <c r="M3" s="28">
+      <c r="M3" s="44">
         <f>IF(OR(E3="",E3=0),"",(F3+G3+H3+I3)/E3)</f>
         <v/>
       </c>
@@ -3590,7 +4819,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n"/>
+      <c r="A4" s="45" t="n"/>
       <c r="B4" s="31" t="n"/>
       <c r="C4" s="31" t="n"/>
       <c r="D4" s="31" t="n"/>
@@ -3602,7 +4831,7 @@
       <c r="J4" s="31" t="n"/>
       <c r="K4" s="31" t="n"/>
       <c r="L4" s="32" t="n"/>
-      <c r="M4" s="28">
+      <c r="M4" s="44">
         <f>IF(OR(E4="",E4=0),"",(F4+G4+H4+I4)/E4)</f>
         <v/>
       </c>
@@ -3612,7 +4841,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n"/>
+      <c r="A5" s="45" t="n"/>
       <c r="B5" s="31" t="n"/>
       <c r="C5" s="31" t="n"/>
       <c r="D5" s="31" t="n"/>
@@ -3624,7 +4853,7 @@
       <c r="J5" s="31" t="n"/>
       <c r="K5" s="31" t="n"/>
       <c r="L5" s="32" t="n"/>
-      <c r="M5" s="28">
+      <c r="M5" s="44">
         <f>IF(OR(E5="",E5=0),"",(F5+G5+H5+I5)/E5)</f>
         <v/>
       </c>
@@ -3634,7 +4863,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="n"/>
+      <c r="A6" s="45" t="n"/>
       <c r="B6" s="31" t="n"/>
       <c r="C6" s="31" t="n"/>
       <c r="D6" s="31" t="n"/>
@@ -3646,7 +4875,7 @@
       <c r="J6" s="31" t="n"/>
       <c r="K6" s="31" t="n"/>
       <c r="L6" s="32" t="n"/>
-      <c r="M6" s="28">
+      <c r="M6" s="44">
         <f>IF(OR(E6="",E6=0),"",(F6+G6+H6+I6)/E6)</f>
         <v/>
       </c>
@@ -3656,7 +4885,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="n"/>
+      <c r="A7" s="45" t="n"/>
       <c r="B7" s="31" t="n"/>
       <c r="C7" s="31" t="n"/>
       <c r="D7" s="31" t="n"/>
@@ -3668,7 +4897,7 @@
       <c r="J7" s="31" t="n"/>
       <c r="K7" s="31" t="n"/>
       <c r="L7" s="32" t="n"/>
-      <c r="M7" s="28">
+      <c r="M7" s="44">
         <f>IF(OR(E7="",E7=0),"",(F7+G7+H7+I7)/E7)</f>
         <v/>
       </c>
@@ -3678,7 +4907,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="n"/>
+      <c r="A8" s="45" t="n"/>
       <c r="B8" s="31" t="n"/>
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="31" t="n"/>
@@ -3690,7 +4919,7 @@
       <c r="J8" s="31" t="n"/>
       <c r="K8" s="31" t="n"/>
       <c r="L8" s="32" t="n"/>
-      <c r="M8" s="28">
+      <c r="M8" s="44">
         <f>IF(OR(E8="",E8=0),"",(F8+G8+H8+I8)/E8)</f>
         <v/>
       </c>
@@ -3700,7 +4929,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="n"/>
+      <c r="A9" s="45" t="n"/>
       <c r="B9" s="31" t="n"/>
       <c r="C9" s="31" t="n"/>
       <c r="D9" s="31" t="n"/>
@@ -3712,7 +4941,7 @@
       <c r="J9" s="31" t="n"/>
       <c r="K9" s="31" t="n"/>
       <c r="L9" s="32" t="n"/>
-      <c r="M9" s="28">
+      <c r="M9" s="44">
         <f>IF(OR(E9="",E9=0),"",(F9+G9+H9+I9)/E9)</f>
         <v/>
       </c>
@@ -3722,7 +4951,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="n"/>
+      <c r="A10" s="45" t="n"/>
       <c r="B10" s="31" t="n"/>
       <c r="C10" s="31" t="n"/>
       <c r="D10" s="31" t="n"/>
@@ -3734,7 +4963,7 @@
       <c r="J10" s="31" t="n"/>
       <c r="K10" s="31" t="n"/>
       <c r="L10" s="32" t="n"/>
-      <c r="M10" s="28">
+      <c r="M10" s="44">
         <f>IF(OR(E10="",E10=0),"",(F10+G10+H10+I10)/E10)</f>
         <v/>
       </c>
@@ -3744,7 +4973,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="n"/>
+      <c r="A11" s="45" t="n"/>
       <c r="B11" s="31" t="n"/>
       <c r="C11" s="31" t="n"/>
       <c r="D11" s="31" t="n"/>
@@ -3756,7 +4985,7 @@
       <c r="J11" s="31" t="n"/>
       <c r="K11" s="31" t="n"/>
       <c r="L11" s="32" t="n"/>
-      <c r="M11" s="28">
+      <c r="M11" s="44">
         <f>IF(OR(E11="",E11=0),"",(F11+G11+H11+I11)/E11)</f>
         <v/>
       </c>
@@ -3766,7 +4995,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="n"/>
+      <c r="A12" s="45" t="n"/>
       <c r="B12" s="31" t="n"/>
       <c r="C12" s="31" t="n"/>
       <c r="D12" s="31" t="n"/>
@@ -3778,7 +5007,7 @@
       <c r="J12" s="31" t="n"/>
       <c r="K12" s="31" t="n"/>
       <c r="L12" s="32" t="n"/>
-      <c r="M12" s="28">
+      <c r="M12" s="44">
         <f>IF(OR(E12="",E12=0),"",(F12+G12+H12+I12)/E12)</f>
         <v/>
       </c>
@@ -3788,7 +5017,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="n"/>
+      <c r="A13" s="45" t="n"/>
       <c r="B13" s="31" t="n"/>
       <c r="C13" s="31" t="n"/>
       <c r="D13" s="31" t="n"/>
@@ -3800,7 +5029,7 @@
       <c r="J13" s="31" t="n"/>
       <c r="K13" s="31" t="n"/>
       <c r="L13" s="32" t="n"/>
-      <c r="M13" s="28">
+      <c r="M13" s="44">
         <f>IF(OR(E13="",E13=0),"",(F13+G13+H13+I13)/E13)</f>
         <v/>
       </c>
@@ -3810,7 +5039,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="n"/>
+      <c r="A14" s="45" t="n"/>
       <c r="B14" s="31" t="n"/>
       <c r="C14" s="31" t="n"/>
       <c r="D14" s="31" t="n"/>
@@ -3822,7 +5051,7 @@
       <c r="J14" s="31" t="n"/>
       <c r="K14" s="31" t="n"/>
       <c r="L14" s="32" t="n"/>
-      <c r="M14" s="28">
+      <c r="M14" s="44">
         <f>IF(OR(E14="",E14=0),"",(F14+G14+H14+I14)/E14)</f>
         <v/>
       </c>
@@ -3832,7 +5061,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="n"/>
+      <c r="A15" s="45" t="n"/>
       <c r="B15" s="31" t="n"/>
       <c r="C15" s="31" t="n"/>
       <c r="D15" s="31" t="n"/>
@@ -3844,7 +5073,7 @@
       <c r="J15" s="31" t="n"/>
       <c r="K15" s="31" t="n"/>
       <c r="L15" s="32" t="n"/>
-      <c r="M15" s="28">
+      <c r="M15" s="44">
         <f>IF(OR(E15="",E15=0),"",(F15+G15+H15+I15)/E15)</f>
         <v/>
       </c>
@@ -3854,7 +5083,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="n"/>
+      <c r="A16" s="45" t="n"/>
       <c r="B16" s="31" t="n"/>
       <c r="C16" s="31" t="n"/>
       <c r="D16" s="31" t="n"/>
@@ -3866,7 +5095,7 @@
       <c r="J16" s="31" t="n"/>
       <c r="K16" s="31" t="n"/>
       <c r="L16" s="32" t="n"/>
-      <c r="M16" s="28">
+      <c r="M16" s="44">
         <f>IF(OR(E16="",E16=0),"",(F16+G16+H16+I16)/E16)</f>
         <v/>
       </c>
@@ -3876,7 +5105,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="n"/>
+      <c r="A17" s="45" t="n"/>
       <c r="B17" s="31" t="n"/>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="31" t="n"/>
@@ -3888,7 +5117,7 @@
       <c r="J17" s="31" t="n"/>
       <c r="K17" s="31" t="n"/>
       <c r="L17" s="32" t="n"/>
-      <c r="M17" s="28">
+      <c r="M17" s="44">
         <f>IF(OR(E17="",E17=0),"",(F17+G17+H17+I17)/E17)</f>
         <v/>
       </c>
@@ -3898,7 +5127,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="30" t="n"/>
+      <c r="A18" s="45" t="n"/>
       <c r="B18" s="31" t="n"/>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="31" t="n"/>
@@ -3910,7 +5139,7 @@
       <c r="J18" s="31" t="n"/>
       <c r="K18" s="31" t="n"/>
       <c r="L18" s="32" t="n"/>
-      <c r="M18" s="28">
+      <c r="M18" s="44">
         <f>IF(OR(E18="",E18=0),"",(F18+G18+H18+I18)/E18)</f>
         <v/>
       </c>
@@ -3920,7 +5149,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="n"/>
+      <c r="A19" s="45" t="n"/>
       <c r="B19" s="31" t="n"/>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="31" t="n"/>
@@ -3932,7 +5161,7 @@
       <c r="J19" s="31" t="n"/>
       <c r="K19" s="31" t="n"/>
       <c r="L19" s="32" t="n"/>
-      <c r="M19" s="28">
+      <c r="M19" s="44">
         <f>IF(OR(E19="",E19=0),"",(F19+G19+H19+I19)/E19)</f>
         <v/>
       </c>
@@ -3942,7 +5171,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="n"/>
+      <c r="A20" s="45" t="n"/>
       <c r="B20" s="31" t="n"/>
       <c r="C20" s="31" t="n"/>
       <c r="D20" s="31" t="n"/>
@@ -3954,7 +5183,7 @@
       <c r="J20" s="31" t="n"/>
       <c r="K20" s="31" t="n"/>
       <c r="L20" s="32" t="n"/>
-      <c r="M20" s="28">
+      <c r="M20" s="44">
         <f>IF(OR(E20="",E20=0),"",(F20+G20+H20+I20)/E20)</f>
         <v/>
       </c>
@@ -3964,7 +5193,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="30" t="n"/>
+      <c r="A21" s="45" t="n"/>
       <c r="B21" s="31" t="n"/>
       <c r="C21" s="31" t="n"/>
       <c r="D21" s="31" t="n"/>
@@ -3976,7 +5205,7 @@
       <c r="J21" s="31" t="n"/>
       <c r="K21" s="31" t="n"/>
       <c r="L21" s="32" t="n"/>
-      <c r="M21" s="28">
+      <c r="M21" s="44">
         <f>IF(OR(E21="",E21=0),"",(F21+G21+H21+I21)/E21)</f>
         <v/>
       </c>
@@ -3986,7 +5215,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="n"/>
+      <c r="A22" s="45" t="n"/>
       <c r="B22" s="31" t="n"/>
       <c r="C22" s="31" t="n"/>
       <c r="D22" s="31" t="n"/>
@@ -3998,7 +5227,7 @@
       <c r="J22" s="31" t="n"/>
       <c r="K22" s="31" t="n"/>
       <c r="L22" s="32" t="n"/>
-      <c r="M22" s="28">
+      <c r="M22" s="44">
         <f>IF(OR(E22="",E22=0),"",(F22+G22+H22+I22)/E22)</f>
         <v/>
       </c>
@@ -4008,7 +5237,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="n"/>
+      <c r="A23" s="45" t="n"/>
       <c r="B23" s="31" t="n"/>
       <c r="C23" s="31" t="n"/>
       <c r="D23" s="31" t="n"/>
@@ -4020,7 +5249,7 @@
       <c r="J23" s="31" t="n"/>
       <c r="K23" s="31" t="n"/>
       <c r="L23" s="32" t="n"/>
-      <c r="M23" s="28">
+      <c r="M23" s="44">
         <f>IF(OR(E23="",E23=0),"",(F23+G23+H23+I23)/E23)</f>
         <v/>
       </c>
@@ -4030,7 +5259,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="30" t="n"/>
+      <c r="A24" s="45" t="n"/>
       <c r="B24" s="31" t="n"/>
       <c r="C24" s="31" t="n"/>
       <c r="D24" s="31" t="n"/>
@@ -4042,7 +5271,7 @@
       <c r="J24" s="31" t="n"/>
       <c r="K24" s="31" t="n"/>
       <c r="L24" s="32" t="n"/>
-      <c r="M24" s="28">
+      <c r="M24" s="44">
         <f>IF(OR(E24="",E24=0),"",(F24+G24+H24+I24)/E24)</f>
         <v/>
       </c>
@@ -4052,7 +5281,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="n"/>
+      <c r="A25" s="45" t="n"/>
       <c r="B25" s="31" t="n"/>
       <c r="C25" s="31" t="n"/>
       <c r="D25" s="31" t="n"/>
@@ -4064,7 +5293,7 @@
       <c r="J25" s="31" t="n"/>
       <c r="K25" s="31" t="n"/>
       <c r="L25" s="32" t="n"/>
-      <c r="M25" s="28">
+      <c r="M25" s="44">
         <f>IF(OR(E25="",E25=0),"",(F25+G25+H25+I25)/E25)</f>
         <v/>
       </c>
@@ -4074,7 +5303,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="30" t="n"/>
+      <c r="A26" s="45" t="n"/>
       <c r="B26" s="31" t="n"/>
       <c r="C26" s="31" t="n"/>
       <c r="D26" s="31" t="n"/>
@@ -4086,7 +5315,7 @@
       <c r="J26" s="31" t="n"/>
       <c r="K26" s="31" t="n"/>
       <c r="L26" s="32" t="n"/>
-      <c r="M26" s="28">
+      <c r="M26" s="44">
         <f>IF(OR(E26="",E26=0),"",(F26+G26+H26+I26)/E26)</f>
         <v/>
       </c>
@@ -4096,7 +5325,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="30" t="n"/>
+      <c r="A27" s="45" t="n"/>
       <c r="B27" s="31" t="n"/>
       <c r="C27" s="31" t="n"/>
       <c r="D27" s="31" t="n"/>
@@ -4108,7 +5337,7 @@
       <c r="J27" s="31" t="n"/>
       <c r="K27" s="31" t="n"/>
       <c r="L27" s="32" t="n"/>
-      <c r="M27" s="28">
+      <c r="M27" s="44">
         <f>IF(OR(E27="",E27=0),"",(F27+G27+H27+I27)/E27)</f>
         <v/>
       </c>
@@ -4118,7 +5347,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="30" t="n"/>
+      <c r="A28" s="45" t="n"/>
       <c r="B28" s="31" t="n"/>
       <c r="C28" s="31" t="n"/>
       <c r="D28" s="31" t="n"/>
@@ -4130,7 +5359,7 @@
       <c r="J28" s="31" t="n"/>
       <c r="K28" s="31" t="n"/>
       <c r="L28" s="32" t="n"/>
-      <c r="M28" s="28">
+      <c r="M28" s="44">
         <f>IF(OR(E28="",E28=0),"",(F28+G28+H28+I28)/E28)</f>
         <v/>
       </c>
@@ -4140,7 +5369,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="30" t="n"/>
+      <c r="A29" s="45" t="n"/>
       <c r="B29" s="31" t="n"/>
       <c r="C29" s="31" t="n"/>
       <c r="D29" s="31" t="n"/>
@@ -4152,7 +5381,7 @@
       <c r="J29" s="31" t="n"/>
       <c r="K29" s="31" t="n"/>
       <c r="L29" s="32" t="n"/>
-      <c r="M29" s="28">
+      <c r="M29" s="44">
         <f>IF(OR(E29="",E29=0),"",(F29+G29+H29+I29)/E29)</f>
         <v/>
       </c>
@@ -4162,7 +5391,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="30" t="n"/>
+      <c r="A30" s="45" t="n"/>
       <c r="B30" s="31" t="n"/>
       <c r="C30" s="31" t="n"/>
       <c r="D30" s="31" t="n"/>
@@ -4174,7 +5403,7 @@
       <c r="J30" s="31" t="n"/>
       <c r="K30" s="31" t="n"/>
       <c r="L30" s="32" t="n"/>
-      <c r="M30" s="28">
+      <c r="M30" s="44">
         <f>IF(OR(E30="",E30=0),"",(F30+G30+H30+I30)/E30)</f>
         <v/>
       </c>
@@ -4184,7 +5413,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="n"/>
+      <c r="A31" s="45" t="n"/>
       <c r="B31" s="31" t="n"/>
       <c r="C31" s="31" t="n"/>
       <c r="D31" s="31" t="n"/>
@@ -4196,7 +5425,7 @@
       <c r="J31" s="31" t="n"/>
       <c r="K31" s="31" t="n"/>
       <c r="L31" s="32" t="n"/>
-      <c r="M31" s="28">
+      <c r="M31" s="44">
         <f>IF(OR(E31="",E31=0),"",(F31+G31+H31+I31)/E31)</f>
         <v/>
       </c>
@@ -4206,7 +5435,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="30" t="n"/>
+      <c r="A32" s="45" t="n"/>
       <c r="B32" s="31" t="n"/>
       <c r="C32" s="31" t="n"/>
       <c r="D32" s="31" t="n"/>
@@ -4218,7 +5447,7 @@
       <c r="J32" s="31" t="n"/>
       <c r="K32" s="31" t="n"/>
       <c r="L32" s="32" t="n"/>
-      <c r="M32" s="28">
+      <c r="M32" s="44">
         <f>IF(OR(E32="",E32=0),"",(F32+G32+H32+I32)/E32)</f>
         <v/>
       </c>
@@ -4267,7 +5496,7 @@
         <f>SUM(L2:L32)</f>
         <v/>
       </c>
-      <c r="M34" s="36">
+      <c r="M34" s="46">
         <f>IF(SUM(E2:E32)=0,"",SUM(F2:I32)/SUM(E2:E32))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add per-video script, scene-by-scene, and real video references to planning sheet
- 3 new columns in Planning 30 Hari: Script (VO/Teks), Scene-by-Scene,
  Video Referensi (real, clickable)
- Each of 30 contents gets full shootable script with timecodes and a
  shot-by-shot scene breakdown
- References mapped to real Kalodata top-performing videos (Men's Underwear
  ID, 30d) by matching format; lifestyle/BTS formats point to TikTok tag refs

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FdFYs9Ji5gfr8VFihGLxdU
</commit_message>
<xml_diff>
--- a/toni-black/toni-black-content-planning.xlsx
+++ b/toni-black/toni-black-content-planning.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="DD MMM YYYY"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +75,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="12">
@@ -135,7 +141,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -157,11 +163,44 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -265,6 +304,10 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2325,7 +2368,7 @@
           <t>Ciri Khas</t>
         </is>
       </c>
-      <c r="E15" s="41" t="n"/>
+      <c r="E15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
@@ -2348,7 +2391,7 @@
           <t>Produk langsung di 3 detik pertama, hashtag agresif (#cdpria #boxerpria #fyp), fokus visual + promo, no intro.</t>
         </is>
       </c>
-      <c r="E16" s="8" t="n"/>
+      <c r="E16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
@@ -2371,7 +2414,7 @@
           <t>Tunjuk bahan (katun/ice silk/seamless), close-up/slow-mo tekstur, angle berbagai sisi, bundle promo.</t>
         </is>
       </c>
-      <c r="E17" s="8" t="n"/>
+      <c r="E17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
@@ -2394,7 +2437,7 @@
           <t>Unboxing excited, review singkat (lembut/adem/nyaman), size chart &amp; pilihan warna, CTA keranjang kuning.</t>
         </is>
       </c>
-      <c r="E18" s="8" t="n"/>
+      <c r="E18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
@@ -2417,7 +2460,7 @@
           <t>AI-generated, hampir 100% dari paid ads, pure product showcase tanpa narasi, biaya produksi rendah.</t>
         </is>
       </c>
-      <c r="E19" s="8" t="n"/>
+      <c r="E19" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -2727,7 +2770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2743,6 +2786,9 @@
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2811,6 +2857,21 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Script (VO / Teks)</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>Scene-by-Scene</t>
+        </is>
+      </c>
+      <c r="P1" s="6" t="inlineStr">
+        <is>
+          <t>Video Referensi (real)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="42" t="n">
@@ -2872,6 +2933,29 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N2" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] VO: "Semua orang bilang kami gila jual celana dalam 100 ribu SATU pcs." | Teks: KATANYA KAMI GILA
+[3-10s] "Padahal alasannya sederhana. Ada tiga."
+[10-30s] "Satu: bahannya micromodal, bukan poliester 15 ribuan. Dua: jahitannya flatlock, nggak bikin lecet. Tiga: tiap unit lolos QC manual." (tunjuk tiap bagian)
+[30-38s] "Kami nggak jual banyak. Kami jual satu yang kamu pakai tiap hari." | Teks: QUIET LUXURY STARTS UNDERNEATH
+CTA: "Follow — kami buktikan satu per satu."</t>
+        </is>
+      </c>
+      <c r="O2" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] MCU founder pegang 1 pcs, eye-contact ke kamera.
+S2 [3-10s] Cut ke b-roll produk di atas meja kayu.
+S3 [10-30s] 3 insert close-up: serat bahan, jahitan flatlock, tangan cek QC.
+S4 [30-38s] Balik ke founder, taruh produk, senyum.
+S5 Endcard logo + handle.</t>
+        </is>
+      </c>
+      <c r="P2" s="48" t="inlineStr">
+        <is>
+          <t>Format talking-head — pelajari confidence &amp; pacing; adaptasi jadi storytelling founder.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="42" t="n">
@@ -2933,6 +3017,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Kalau 3 dari 5 ini ada di CD kamu, buang. Sekarang." | Teks: 5 TANDA HARUS DIBUANG
+[3-28s] 1. Karet melar. 2. Kain menipis/nerawang. 3. Warna kusam permanen. 4. Bau nggak hilang walau dicuci. 5. Umur lebih dari setahun. (tiap poin 4-5 detik + angka besar)
+[28-33s] "Kena berapa poin? Komen di bawah."</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook host to-camera.
+S2-S6 lima insert b-roll CD lama (blur) + angka overlay tiap tanda.
+S7 host CTA + gesture komen.</t>
+        </is>
+      </c>
+      <c r="P3" s="48" t="inlineStr">
+        <is>
+          <t>Format short-listicle — pelajari hook 3 detik &amp; text-overlay cepat.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="42" t="n">
@@ -2994,6 +3097,28 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "CD 100 ribu vs 10 ribu. Kita tarik sampai salah satu nyerah."
+[3-20s] "Dua-duanya ditarik dengan beban sama." (tarik pelan, makro serat)
+[20-30s] "Yang murah melar dan nggak balik. Yang ini balik lagi." (tunjuk recovery)
+[30-35s] "Kualitas kerasa dari tarikan pertama. Cek keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook dua produk di tangan.
+S2 [3-20s] Wide dua tangan menarik bersamaan.
+S3 makro serat saat ditarik.
+S4 [20-30s] Side-by-side hasil recovery.
+S5 endcard CTA.</t>
+        </is>
+      </c>
+      <c r="P4" s="48" t="inlineStr">
+        <is>
+          <t>Demo elastis/tarik bahan — pelajari teknik demo side-by-side.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="42" t="n">
@@ -3055,6 +3180,27 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Area intim gampang gatal &amp; lembab? Bukan karena jorok."
+[3-12s] "Penyebabnya: bahan nggak breathable, lembab kejebak, gesekan jahitan."
+[12-28s] "Solusinya bukan bedak. Tapi pilih bahan yang bisa 'napas' dan jahitan yang halus." (tunjuk sampel bahan)
+[28-33s] "Share ke temanmu yang sering ngeluh."</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Host to-cam, ekspresi serius.
+S2 [3-12s] Grafis sederhana penyebab + b-roll kulit/kain (aman).
+S3 [12-28s] Insert sampel bahan breathable vs tidak.
+S4 CTA share.</t>
+        </is>
+      </c>
+      <c r="P5" s="48" t="inlineStr">
+        <is>
+          <t>Edukasi + b-roll bahan — pelajari struktur talking-head 60-80 detik.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="42" t="n">
@@ -3116,6 +3262,27 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Bukan jam. Bukan sepatu. Hal pertama yang bikin cowok keliatan mahal itu ini."
+[3-22s] "Tiga hal yang orang lain nggak lihat: wangi, kuku rapi, dan dalaman berkualitas."
+[22-30s] "Kemewahan yang kamu rasakan sendiri." (flat lay produk)
+[30-35s] "Mulai dari yang paling dalam. Link di bio."</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Host to-cam berpakaian rapi.
+S2 [3-22s] 3 b-roll: parfum, gunting kuku, laci produk.
+S3 flat lay produk elegan.
+S4 endcard.</t>
+        </is>
+      </c>
+      <c r="P6" s="48" t="inlineStr">
+        <is>
+          <t>Tone premium/quiet-luxury — pelajari mood &amp; warna. (referensi lifestyle di luar kategori CD)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="42" t="n">
@@ -3177,6 +3344,27 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Tuang air ke dua kain ini. Lihat mana yang 'minum' duluan."
+[3-18s] (slow-mo) air di kain murah menggenang; di kain Toni Black langsung menyerap.
+[18-26s] "Ini yang namanya moisture-wicking. Kering = kulit sehat."
+[26-31s] "Kulitmu tahu bedanya. Keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook dua potong kain berlabel.
+S2 [3-18s] Makro slow-mo tetes air di dua kain.
+S3 [18-26s] Split-screen hasil serap.
+S4 endcard CTA.</t>
+        </is>
+      </c>
+      <c r="P7" s="48" t="inlineStr">
+        <is>
+          <t>Demo close-up satisfying — pelajari framing makro &amp; slow-mo.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="42" t="n">
@@ -3238,6 +3426,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] VO: "Hal paling mahal yang dia pakai hari ini... nggak keliatan." | Teks sama.
+[3-22s] (sinematik, tanpa dialog) rutinitas pagi: kopi, skincare, kancing kemeja, buka laci berisi CD tersusun rapi (produk dilipat, tidak dipakai di kamera).
+[22-28s] Teks: UPGRADE DIMULAI DARI DALAM. | "Link di bio."</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] CU wajah/tangan + teks hook.
+S2 [3-22s] Montase 4-5 shot cinematic pagi, gerak kamera halus.
+S3 CU laci produk rapi.
+S4 endcard teks.</t>
+        </is>
+      </c>
+      <c r="P8" s="48" t="inlineStr">
+        <is>
+          <t>Format POV morning-routine/quiet-luxury (di luar kategori CD) — pelajari sinematografi &amp; mood.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="42" t="n">
@@ -3299,6 +3507,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Bahan CD kamu menentukan kesehatan kulitmu. Serius."
+[3-25s] Pegang 3 sampel: poliester murah (panas), katun biasa (nyerap tapi lama kering), micromodal premium (lembut + breathable). Jelaskan beda serat &amp; sirkulasi udara.
+[25-30s] "Save sebelum beli CD lagi."</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Host pegang 3 sampel.
+S2 [3-25s] Insert makro tiap kain + label nama bahan.
+S3 demo remas/tiup untuk breathability.
+S4 CTA save.</t>
+        </is>
+      </c>
+      <c r="P9" s="48" t="inlineStr">
+        <is>
+          <t>Perbandingan bahan/talking-head — pelajari cara tunjuk detail material.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="42" t="n">
@@ -3360,6 +3588,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Ini alasan kenapa 1 pcs harganya 100 ribu. Kita bedah."
+[3-45s] Bedah per bagian: gramasi bahan (timbang), jahitan flatlock (makro), waistband tenun (tarik), karet premium. Bandingkan diam-diam dengan CD murah yang juga dibedah.
+[45-55s] "Sekarang kamu tahu bayar untuk apa. Link di bio."</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook produk utuh + gunting.
+S2-S5 empat insert makro tiap komponen (bahan, jahitan, waistband, karet).
+S6 side-by-side vs CD murah terbedah.
+S7 endcard.</t>
+        </is>
+      </c>
+      <c r="P10" s="48" t="inlineStr">
+        <is>
+          <t>Demo detail bahan/jahitan 60-80 detik — GPM tertinggi. Pelajari struktur demo Uomo.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="42" t="n">
@@ -3421,6 +3669,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Yang nggak lolos QC, nggak kami diskon. Kami gunting."
+[3-25s] Proses QC: cek jahitan, tarik karet, terawang kain → temukan cacat → gunting produk gagal di depan kamera.
+[25-32s] "Ini standar yang kamu bayar. Follow untuk BTS lain."</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] CU tangan pegang produk + gunting.
+S2 [3-25s] Beberapa insert proses cek QC di meja.
+S3 momen gunting (satisfying).
+S4 endcard.</t>
+        </is>
+      </c>
+      <c r="P11" s="48" t="inlineStr">
+        <is>
+          <t>Format BTS/QC (di luar kategori CD) — pelajari teknik close-up proses dari demo Uomo.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="42" t="n">
@@ -3482,6 +3750,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Kamu pakai CD yang sama lebih dari setahun? Dengerin dulu."
+[3-20s] "Menurut dermatolog, CD idealnya dirotasi dan diganti total tiap 6-12 bulan. Kain lama menyimpan bakteri walau sudah dicuci."
+[20-27s] "Cek laci kamu malam ini."</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Host to-cam.
+S2 [3-20s] Text overlay angka '6-12 bulan' + b-roll laci CD.
+S3 CTA.</t>
+        </is>
+      </c>
+      <c r="P12" s="48" t="inlineStr">
+        <is>
+          <t>Talking-head edukasi + otoritas — pelajari hook 3 detik.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="42" t="n">
@@ -3543,6 +3830,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Kado buat cowok itu gampang. Yang susah: kado yang dia PAKAI."
+[3-22s] "Parfum? Numpuk. Dompet? Udah punya. Tapi celana dalam premium — dipakai TIAP hari." (tunjuk gift box)
+[22-30s] Reaksi unboxing pasangan. "Tag pasanganmu. Gift box di keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Talent perempuan to-cam pegang gift box.
+S2 [3-22s] B-roll kado 'gagal' vs gift box Toni Black.
+S3 [22-30s] Reaksi unboxing.
+S4 endcard CTA tag.</t>
+        </is>
+      </c>
+      <c r="P13" s="48" t="inlineStr">
+        <is>
+          <t>Testimoni/gift warm-tone — pelajari cara review &amp; CTA gift.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="42" t="n">
@@ -3604,6 +3911,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>(Tanpa dialog — full ASMR) Teks awal: "Kado terbaik itu yang dipakai tiap hari."
+Urutan suara: buka sleeve box → tissue paper → angkat produk terlipat → kartu ucapan → tutup box.
+Teks akhir: "Kirim ke dia yang perlu upgrade."</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-4s] CU tangan buka box + teks.
+S2-S4 makro tiap tahap unboxing, suara asli dominan.
+S5 produk final di frame + teks CTA.</t>
+        </is>
+      </c>
+      <c r="P14" s="48" t="inlineStr">
+        <is>
+          <t>Format ASMR unboxing — pelajari pacing &amp; makro (referensi unboxing kategori + #asmrunboxing).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="42" t="n">
@@ -3665,6 +3991,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Aku beliin suamiku celana dalam 100 ribu. Reaksinya di luar dugaan."
+[3-25s] "Awalnya dia protes 'kemahalan'. Seminggu kemudian... dia minta dibeliin lagi." (screenshot chat asli, dengan izin)
+[25-30s] "Coba dulu 1 pcs. Keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] UGC istri to-cam (natural, handheld).
+S2 [3-25s] Insert screenshot chat + b-roll produk.
+S3 CTA.</t>
+        </is>
+      </c>
+      <c r="P15" s="48" t="inlineStr">
+        <is>
+          <t>UGC testimoni natural — pelajari gaya bicara jujur non-scripted.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="42" t="n">
@@ -3726,6 +4071,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Kesalahan nomor 2 dilakukan 90% pria Indonesia."
+[3-24s] 1. Beli karena murah per lusin. 2. Salah ukuran (ikut ukuran kaos). 3. Nggak lihat bahan. (tiap poin solusi singkat)
+[24-29s] "Kamu pernah yang mana? Komen."</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook host to-cam.
+S2-S4 tiga insert ilustrasi tiap kesalahan + angka.
+S5 CTA komen.</t>
+        </is>
+      </c>
+      <c r="P16" s="48" t="inlineStr">
+        <is>
+          <t>Short-listicle cepat — pelajari ritme potongan per poin.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="42" t="n">
@@ -3787,6 +4151,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Kalau uap aja nggak bisa lewat, gimana kulitmu bisa napas?"
+[3-20s] Uap/hairdryer di balik dua kain: kain murah menahan uap; Toni Black tembus. "Ini bedanya breathable."
+[20-26s] "Kulit juga butuh napas. Link di bio."</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook dua kain di ring/frame.
+S2 [3-20s] Uap dari bawah, kamera samping, lihat tembus/tidak.
+S3 close-up perbandingan.
+S4 endcard.</t>
+        </is>
+      </c>
+      <c r="P17" s="48" t="inlineStr">
+        <is>
+          <t>Demo eksperimen — pelajari framing demo produk 60-70 detik.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="42" t="n">
@@ -3848,6 +4232,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Umur 30 ke atas, upgrade dulu barang yang kamu pakai TIAP HARI."
+[3-24s] "Konsep cost-per-wear: barang harian premium lebih masuk akal daripada barang pamer yang jarang dipakai. Kasur, sepatu harian... dan celana dalam."
+[24-30s] "Hitung cost-per-wear-mu. Link di bio."</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Host to-cam.
+S2 [3-24s] B-roll lifestyle + grafis hitung cost-per-wear.
+S3 endcard.</t>
+        </is>
+      </c>
+      <c r="P18" s="48" t="inlineStr">
+        <is>
+          <t>Talking-head premium + b-roll — pelajari tone aspiratif.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="42" t="n">
@@ -3909,6 +4312,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Katanya CD ketat itu bahaya. Mitos atau fakta?"
+[3-22s] "Yang penting bukan ketat atau longgar — tapi bahan breathable dan ukuran yang pas. Ini cara cek ukuranmu." (tunjuk size chart)
+[22-28s] "Save untuk referensi ukuran."</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook host, teks MITOS / FAKTA.
+S2 [3-22s] Insert size chart + demo ukur.
+S3 CTA save.</t>
+        </is>
+      </c>
+      <c r="P19" s="48" t="inlineStr">
+        <is>
+          <t>Mitos-fakta/short edukasi — pelajari hook singkat.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="42" t="n">
@@ -3970,6 +4392,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] (Reply to Comment) Screenshot komen: 'mending 10 pcs 100rb' → "Oke, kita hitung bareng."
+[3-25s] "CD murah rusak 2 bulan. Premium tahan 1,5-2 tahun. Bagi harga per hari... yang premium justru lebih murah." (grafik kalkulator on-screen)
+[25-30s] "Masih tim borongan? Komen di bawah."</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Tempel screenshot komen (fitur Reply) + host.
+S2 [3-25s] Animasi hitung cost-per-wear.
+S3 host senyum, tanpa defensif.</t>
+        </is>
+      </c>
+      <c r="P20" s="48" t="inlineStr">
+        <is>
+          <t>Gunakan fitur TikTok 'Reply to Comment' — pelajari format di #replytocomment.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="42" t="n">
@@ -4031,6 +4472,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Perbedaan 100 ribu itu ada di detail yang nggak pernah kamu perhatiin."
+[3-25s] (makro slow-mo) jahitan flatlock anti-gesek, tenunan waistband, label tanpa jahitan gatal. Side-by-side dengan jahitan CD murah yang kasar.
+[25-30s] "Detail itu mahal. Link di bio."</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook produk + teks.
+S2-S4 makro tiga detail (jahitan, waistband, label).
+S5 side-by-side vs murah.
+S6 endcard.</t>
+        </is>
+      </c>
+      <c r="P21" s="48" t="inlineStr">
+        <is>
+          <t>Makro detail produk — pelajari close-up demo Uomo.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="42" t="n">
@@ -4092,6 +4553,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Business trip 3 hari, 1 tas kabin. Yang pertama masuk?"
+[3-22s] Packing rapi: kemeja digulung, pouch skincare, lalu pouch dalaman premium Toni Black masuk duluan.
+[22-28s] "Travel kit ada di keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook tas kabin terbuka.
+S2 [3-22s] Time-lapse/ritmis packing tiap item.
+S3 CU pouch produk.
+S4 endcard.</t>
+        </is>
+      </c>
+      <c r="P22" s="48" t="inlineStr">
+        <is>
+          <t>Format packing video (di luar kategori CD) — pelajari ritme di #packing.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="42" t="n">
@@ -4153,6 +4634,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Barang 100 ribu dirawatnya beda. Ini caranya."
+[3-24s] 3 aturan: cuci lembut/tangan, jangan pengering panas, jemur terbalik tanpa matahari langsung. Bonus: cara melipat ala retail.
+[24-30s] "Save biar investasimu awet 2 tahun."</t>
+        </is>
+      </c>
+      <c r="O23" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Host pegang produk.
+S2-S4 tiga insert langkah perawatan.
+S5 demo lipat rapi.
+S6 CTA save.</t>
+        </is>
+      </c>
+      <c r="P23" s="48" t="inlineStr">
+        <is>
+          <t>Tutorial singkat/talking-head — pelajari struktur how-to.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="42" t="n">
@@ -4214,6 +4715,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "CD ini sudah dicuci 30 kali. Ini bentuknya sekarang."
+[3-22s] Bandingkan unit 30x cuci vs unit baru: warna, karet, bentuk. "Nyaris nggak ada beda." (timelapse dokumentasi cuci)
+[22-28s] "Ini yang kamu bayar. Keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O24" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook dua unit di tangan.
+S2 [3-22s] Timelapse cuci + side-by-side.
+S3 CU karet &amp; warna.
+S4 endcard.</t>
+        </is>
+      </c>
+      <c r="P24" s="48" t="inlineStr">
+        <is>
+          <t>Before/after demo durability — pelajari framing demo produk.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="42" t="n">
@@ -4275,6 +4796,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Kata mereka yang sudah pindah ke Toni Black:"
+[3-24s] Kompilasi 3 screenshot review bintang 5 + voice over highlight ('lembut', 'adem', 'nggak balik lagi ke yang murah').
+[24-30s] "Buktikan sendiri. Keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O25" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook teks + b-roll produk.
+S2-S4 tiga kartu review animasi masuk.
+S5 endcard CTA.</t>
+        </is>
+      </c>
+      <c r="P25" s="48" t="inlineStr">
+        <is>
+          <t>Kompilasi testimoni/review — pelajari tone testimoni KASOGI.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="42" t="n">
@@ -4336,6 +4876,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N26" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Isi tas gym pria yang rapi. Nomor 4 sering dilupakan."
+[3-24s] Sepatu, handuk, skincare mini, lalu CD ganti Toni Black (poin edukasi: keringat = lembab, wajib bawa ganti).
+[24-30s] "Jangan skip nomor 4. Link di bio."</t>
+        </is>
+      </c>
+      <c r="O26" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook tas gym + teks.
+S2 [3-24s] Keluarkan item satu-satu + angka overlay.
+S3 CU produk 'nomor 4'.
+S4 endcard.</t>
+        </is>
+      </c>
+      <c r="P26" s="48" t="inlineStr">
+        <is>
+          <t>Format what's-in-my-bag (di luar kategori CD) — pelajari ritme di #whatsinmygymbag.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="42" t="n">
@@ -4397,6 +4957,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Punya CD banyak itu bukan boros. Ini hitungannya."
+[3-22s] "Sistem rotasi 7+ pcs: tiap kain 'istirahat' setelah dipakai jadi lebih awet, dan kamu selalu punya yang kering." (tunjuk laci tersusun)
+[22-30s] "Lengkapi rotasimu. Bundle hemat di keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O27" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook laci penuh CD rapi.
+S2 [3-22s] Grafis rotasi 7 hari + b-roll.
+S3 CTA bundle.</t>
+        </is>
+      </c>
+      <c r="P27" s="48" t="inlineStr">
+        <is>
+          <t>Edukasi + soft-sell paket — pelajari cara jelaskan value bundle.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="42" t="n">
@@ -4458,6 +5037,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N28" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "100 ribu itu bukan harga kain. Ini prosesnya."
+[3-30s] Perjalanan produk: pilih kain → cutting → jahit → QC → packing. 5-6 detik per tahap + text overlay nama tahap.
+[30-36s] "Sekarang kamu tahu prosesnya. Follow untuk BTS lain."</t>
+        </is>
+      </c>
+      <c r="O28" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook gulungan kain/workshop.
+S2-S6 lima shot tiap tahap produksi.
+S7 endcard.</t>
+        </is>
+      </c>
+      <c r="P28" s="48" t="inlineStr">
+        <is>
+          <t>Format BTS produksi (di luar kategori CD) — pelajari close-up proses dari demo Uomo.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="42" t="n">
@@ -4519,6 +5117,25 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Ada alasannya kenapa CD terbaik di dunia kebanyakan warna gelap."
+[3-20s] "Noda &amp; kusam nggak keliatan, terlihat baru lebih lama, dan netral di balik semua outfit." (tunjuk lini warna)
+[20-26s] "Tim hitam atau tim navy? Komen."</t>
+        </is>
+      </c>
+      <c r="O29" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook host + flat lay warna gelap.
+S2 [3-20s] B-roll produk beberapa warna.
+S3 CTA komen.</t>
+        </is>
+      </c>
+      <c r="P29" s="48" t="inlineStr">
+        <is>
+          <t>Fun-fact/short edukasi — pelajari hook singkat + text overlay.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="42" t="n">
@@ -4580,6 +5197,26 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N30" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Kain CD itu ada 'kelasnya'. Kita timbang biar jujur."
+[3-22s] Timbang kain CD murah vs Toni Black (ukuran sama). "Gramasi lebih tinggi = kain lebih padat &amp; tahan lama. Namanya GSM."
+[22-28s] "Sekarang kamu ngerti GSM. Link di bio."</t>
+        </is>
+      </c>
+      <c r="O30" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook timbangan digital + kain.
+S2 [3-22s] Timbang dua kain, CU angka.
+S3 grafik GSM.
+S4 endcard.</t>
+        </is>
+      </c>
+      <c r="P30" s="48" t="inlineStr">
+        <is>
+          <t>Demo eksperimen/timbangan — pelajari close-up satisfying.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="42" t="n">
@@ -4641,8 +5278,59 @@
           <t>Ide</t>
         </is>
       </c>
+      <c r="N31" s="8" t="inlineStr">
+        <is>
+          <t>[0-3s] "Gajian sudah masuk. Upgrade dulu barang yang kamu pakai TIAP HARI."
+[3-20s] Recap cuplikan demo terbaik bulan ini (stretch test, serap air) + tawaran bundle gift box edisi gajian.
+[20-28s] "LIVE malam ini jam 8. Nyalakan pengingat + cek keranjang kuning."</t>
+        </is>
+      </c>
+      <c r="O31" s="8" t="inlineStr">
+        <is>
+          <t>S1 [0-3s] Hook host energik + teks GAJIAN.
+S2 [3-20s] Montase cuplikan demo + gift box.
+S3 [20-28s] Endcard jadwal LIVE + CTA.</t>
+        </is>
+      </c>
+      <c r="P31" s="48" t="inlineStr">
+        <is>
+          <t>Short promo momen payday + transisi ke LIVE — pelajari CTA payday. (live: studi @ryan.outfitness &amp; @ck_underwear_store)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId30"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remap references to scene-matched videos; remove live streaming
- Video Referensi column now points to videos that mirror each script/scene
  (stretch test, water-absorption test, ASMR unboxing, dermatologist edu,
  care/wash tutorial, quiet luxury POV, packing, gym bag) instead of random
  top-sellers
- Content #30 reworked: payday video promo, live streaming removed
- Strategy doc: live shopping marked as postponed (video-first for now)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FdFYs9Ji5gfr8VFihGLxdU
</commit_message>
<xml_diff>
--- a/toni-black/toni-black-content-planning.xlsx
+++ b/toni-black/toni-black-content-planning.xlsx
@@ -2953,7 +2953,7 @@
       </c>
       <c r="P2" s="48" t="inlineStr">
         <is>
-          <t>Format talking-head — pelajari confidence &amp; pacing; adaptasi jadi storytelling founder.</t>
+          <t>Belum ada video founder di kategori CD (white space). Pelajari pacing premium: P3_QuietLuxury_OldMoney / P2 short premium. Konsep brand-story: SilkCut/Manmade.</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="P3" s="48" t="inlineStr">
         <is>
-          <t>Format short-listicle — pelajari hook 3 detik &amp; text-overlay cepat.</t>
+          <t>Scene match: P1_EdukasiKesehatan_DokterKulit_doctorsooj (listicle kesehatan underwear).</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="P4" s="48" t="inlineStr">
         <is>
-          <t>Demo elastis/tarik bahan — pelajari teknik demo side-by-side.</t>
+          <t>Scene match: P2_StretchTest_ElastisBoxer_harlook (tarik/elastis boxer).</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="P5" s="48" t="inlineStr">
         <is>
-          <t>Edukasi + b-roll bahan — pelajari struktur talking-head 60-80 detik.</t>
+          <t>Scene match: P1_EdukasiKesehatan_DokterKulit_doctorsooj (underwear &amp; masalah kulit — dermatolog).</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="P6" s="48" t="inlineStr">
         <is>
-          <t>Tone premium/quiet-luxury — pelajari mood &amp; warna. (referensi lifestyle di luar kategori CD)</t>
+          <t>Scene match: P3_QuietLuxury_OldMoney_shaynicolexo (tone premium/quiet luxury).</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="P7" s="48" t="inlineStr">
         <is>
-          <t>Demo close-up satisfying — pelajari framing makro &amp; slow-mo.</t>
+          <t>Scene match: P2_WaterTest_SerapAir_bedsure (tuang air ke kain — moisture wicking).</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="P8" s="48" t="inlineStr">
         <is>
-          <t>Format POV morning-routine/quiet-luxury (di luar kategori CD) — pelajari sinematografi &amp; mood.</t>
+          <t>Scene match: P3_QuietLuxury_OldMoney_shaynicolexo (POV/mood morning routine premium).</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="P9" s="48" t="inlineStr">
         <is>
-          <t>Perbandingan bahan/talking-head — pelajari cara tunjuk detail material.</t>
+          <t>Scene match: P1P2_BahanCompare_MoistureWicking_chezcolleen (bandingkan bahan katun vs modal).</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="P10" s="48" t="inlineStr">
         <is>
-          <t>Demo detail bahan/jahitan 60-80 detik — GPM tertinggi. Pelajari struktur demo Uomo.</t>
+          <t>Scene match: P2_DemoProduk_Uomo (demo detail bahan/jahitan — in-category).</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="P11" s="48" t="inlineStr">
         <is>
-          <t>Format BTS/QC (di luar kategori CD) — pelajari teknik close-up proses dari demo Uomo.</t>
+          <t>Adaptasi BTS/QC dari P2_DemoProduk_Uomo (teknik close-up proses). Belum ada video QC di kategori.</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="P12" s="48" t="inlineStr">
         <is>
-          <t>Talking-head edukasi + otoritas — pelajari hook 3 detik.</t>
+          <t>Scene match: P1_EdukasiKesehatan_DokterKulit_doctorsooj (umur/ganti underwear — dermatolog).</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="P13" s="48" t="inlineStr">
         <is>
-          <t>Testimoni/gift warm-tone — pelajari cara review &amp; CTA gift.</t>
+          <t>Angle gift: adaptasi tone review P5_Testimoni_KASOGI. Belum ada video gift khusus di kategori.</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="P14" s="48" t="inlineStr">
         <is>
-          <t>Format ASMR unboxing — pelajari pacing &amp; makro (referensi unboxing kategori + #asmrunboxing).</t>
+          <t>Scene match: P2_ASMRUnboxing_Packaging_theselfdefense (ASMR unboxing/packing).</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4007,7 @@
       </c>
       <c r="P15" s="48" t="inlineStr">
         <is>
-          <t>UGC testimoni natural — pelajari gaya bicara jujur non-scripted.</t>
+          <t>Scene match: P5_Testimoni_KASOGI (testimoni jujur, gaya natural — in-category).</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="P16" s="48" t="inlineStr">
         <is>
-          <t>Short-listicle cepat — pelajari ritme potongan per poin.</t>
+          <t>Scene match: P1_EdukasiKesehatan_DokterKulit_doctorsooj (listicle kesalahan/kesehatan).</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="P17" s="48" t="inlineStr">
         <is>
-          <t>Demo eksperimen — pelajari framing demo produk 60-70 detik.</t>
+          <t>Adaptasi dari P2_WaterTest_SerapAir_bedsure (tes fabric → adaptasi ke tes udara/uap).</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="P18" s="48" t="inlineStr">
         <is>
-          <t>Talking-head premium + b-roll — pelajari tone aspiratif.</t>
+          <t>Scene match: P3_QuietLuxury_OldMoney_shaynicolexo (aspirasi/quiet luxury).</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="P19" s="48" t="inlineStr">
         <is>
-          <t>Mitos-fakta/short edukasi — pelajari hook singkat.</t>
+          <t>Scene match: P1_EdukasiKesehatan_DokterKulit_doctorsooj (mitos-fakta gaya dermatolog).</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="P20" s="48" t="inlineStr">
         <is>
-          <t>Gunakan fitur TikTok 'Reply to Comment' — pelajari format di #replytocomment.</t>
+          <t>Format 'Reply to Comment' (fitur TikTok), bukan video tunggal. Pelajari di tag #replytocomment.</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="P21" s="48" t="inlineStr">
         <is>
-          <t>Makro detail produk — pelajari close-up demo Uomo.</t>
+          <t>Scene match: P2_DemoProduk_Uomo (makro detail jahitan/waistband — in-category).</t>
         </is>
       </c>
     </row>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="P22" s="48" t="inlineStr">
         <is>
-          <t>Format packing video (di luar kategori CD) — pelajari ritme di #packing.</t>
+          <t>Scene match: P3_PackingVideo_Koper_armanidex (packing koper).</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="P23" s="48" t="inlineStr">
         <is>
-          <t>Tutorial singkat/talking-head — pelajari struktur how-to.</t>
+          <t>Scene match: P1_CaraRawat_CuciUnderwear_sisterpledge (cara cuci/rawat underwear).</t>
         </is>
       </c>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="P24" s="48" t="inlineStr">
         <is>
-          <t>Before/after demo durability — pelajari framing demo produk.</t>
+          <t>Adaptasi dari P1_CaraRawat_CuciUnderwear_sisterpledge (before/after durability cuci).</t>
         </is>
       </c>
     </row>
@@ -4812,7 +4812,7 @@
       </c>
       <c r="P25" s="48" t="inlineStr">
         <is>
-          <t>Kompilasi testimoni/review — pelajari tone testimoni KASOGI.</t>
+          <t>Scene match: P5_Testimoni_KASOGI (kompilasi review/testimoni — in-category).</t>
         </is>
       </c>
     </row>
@@ -4893,7 +4893,7 @@
       </c>
       <c r="P26" s="48" t="inlineStr">
         <is>
-          <t>Format what's-in-my-bag (di luar kategori CD) — pelajari ritme di #whatsinmygymbag.</t>
+          <t>Scene match: P3_GymBag_Essentials_alexnicoll (what's in my gym bag pria).</t>
         </is>
       </c>
     </row>
@@ -4973,7 +4973,7 @@
       </c>
       <c r="P27" s="48" t="inlineStr">
         <is>
-          <t>Edukasi + soft-sell paket — pelajari cara jelaskan value bundle.</t>
+          <t>Scene match: P1_PromoPaket_Davina (jelaskan value paket/rotasi — in-category).</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="P28" s="48" t="inlineStr">
         <is>
-          <t>Format BTS produksi (di luar kategori CD) — pelajari close-up proses dari demo Uomo.</t>
+          <t>Adaptasi BTS produksi dari P2_DemoProduk_Uomo (close-up proses). Belum ada di kategori.</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="P29" s="48" t="inlineStr">
         <is>
-          <t>Fun-fact/short edukasi — pelajari hook singkat + text overlay.</t>
+          <t>Scene match: P1_EdukasiKesehatan_DokterKulit_doctorsooj (fun-fact edukasi talking-head).</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="P30" s="48" t="inlineStr">
         <is>
-          <t>Demo eksperimen/timbangan — pelajari close-up satisfying.</t>
+          <t>Adaptasi dari P1P2_BahanCompare_MoistureWicking_chezcolleen (bandingkan/timbang bahan GSM).</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Gajian sudah masuk — saatnya gift box (soft launch LIVE)</t>
+          <t>Gajian sudah masuk — upgrade harian (gift box edisi gajian)</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -5244,17 +5244,17 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>Promo momen gajian</t>
+          <t>Short promo momen payday</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Recap value 1 bulan konten (cuplikan demo terbaik) → tawaran bundle gift box edisi gajian → umumkan jadwal LIVE perdana malam ini.</t>
+          <t>Recap cuplikan demo terbaik bulan ini (stretch test, serap air) + tawaran bundle gift box edisi gajian → arahkan ke keranjang kuning.</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>LIVE malam ini jam 8. Nyalakan pengingat + cek keranjang kuning.</t>
+          <t>Checkout gift box edisi gajian di keranjang kuning.</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
@@ -5264,12 +5264,12 @@
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>#ToniBlack #CelanaDalamPria #UnderwearPria #Gajian #TikTokShop #LiveShopping</t>
+          <t>#ToniBlack #CelanaDalamPria #UnderwearPria #Gajian #TikTokShop</t>
         </is>
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>Cuplikan konten lama, gift box, host live</t>
+          <t>Cuplikan konten lama, gift box, host</t>
         </is>
       </c>
       <c r="L31" s="20" t="inlineStr"/>
@@ -5281,20 +5281,20 @@
       <c r="N31" s="8" t="inlineStr">
         <is>
           <t>[0-3s] "Gajian sudah masuk. Upgrade dulu barang yang kamu pakai TIAP HARI."
-[3-20s] Recap cuplikan demo terbaik bulan ini (stretch test, serap air) + tawaran bundle gift box edisi gajian.
-[20-28s] "LIVE malam ini jam 8. Nyalakan pengingat + cek keranjang kuning."</t>
+[3-18s] Recap cuplikan demo terbaik bulan ini (stretch test, tes serap air) + tunjukkan bundle gift box edisi gajian.
+[18-25s] "Checkout gift box edisi gajian sekarang di keranjang kuning."</t>
         </is>
       </c>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook host energik + teks GAJIAN.
-S2 [3-20s] Montase cuplikan demo + gift box.
-S3 [20-28s] Endcard jadwal LIVE + CTA.</t>
+          <t>S1 [0-3s] Host energik + teks GAJIAN.
+S2 [3-18s] Montase cuplikan demo + gift box.
+S3 [18-25s] Endcard produk + CTA keranjang kuning.</t>
         </is>
       </c>
       <c r="P31" s="48" t="inlineStr">
         <is>
-          <t>Short promo momen payday + transisi ke LIVE — pelajari CTA payday. (live: studi @ryan.outfitness &amp; @ck_underwear_store)</t>
+          <t>Scene match: P5_ShortPromo_SultanKalisari (short promo momen payday — TANPA live).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap all scripts/scenes at 15s; enforce no live streaming
- Rewrote all 30 scripts and scene breakdowns to <=15 seconds (ultra-short)
- Verified no stray live-streaming references remain
- Strategy doc: max duration updated to 15s

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FdFYs9Ji5gfr8VFihGLxdU
</commit_message>
<xml_diff>
--- a/toni-black/toni-black-content-planning.xlsx
+++ b/toni-black/toni-black-content-planning.xlsx
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Founder talking head</t>
+          <t>Founder talking head (≤15 dtk)</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -2935,20 +2935,16 @@
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] VO: "Semua orang bilang kami gila jual celana dalam 100 ribu SATU pcs." | Teks: KATANYA KAMI GILA
-[3-10s] "Padahal alasannya sederhana. Ada tiga."
-[10-30s] "Satu: bahannya micromodal, bukan poliester 15 ribuan. Dua: jahitannya flatlock, nggak bikin lecet. Tiga: tiap unit lolos QC manual." (tunjuk tiap bagian)
-[30-38s] "Kami nggak jual banyak. Kami jual satu yang kamu pakai tiap hari." | Teks: QUIET LUXURY STARTS UNDERNEATH
-CTA: "Follow — kami buktikan satu per satu."</t>
+          <t>[0-2s] "Semua bilang kami gila jual CD 100 ribu SATU pcs."
+[2-12s] "Micromodal premium, jahitan flatlock anti-lecet, tiap unit lolos QC. Bukan 15 ribuan."
+[12-15s] "Quiet luxury starts underneath. Follow."</t>
         </is>
       </c>
       <c r="O2" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] MCU founder pegang 1 pcs, eye-contact ke kamera.
-S2 [3-10s] Cut ke b-roll produk di atas meja kayu.
-S3 [10-30s] 3 insert close-up: serat bahan, jahitan flatlock, tangan cek QC.
-S4 [30-38s] Balik ke founder, taruh produk, senyum.
-S5 Endcard logo + handle.</t>
+          <t>S1 [0-2s] Founder pegang 1 pcs, eye-contact.
+S2 [2-12s] 3 insert kilat: bahan, jahitan, QC.
+S3 [12-15s] Endcard logo + follow.</t>
         </is>
       </c>
       <c r="P2" s="48" t="inlineStr">
@@ -2983,7 +2979,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Talking head + listicle</t>
+          <t>Talking head + listicle (≤15 dtk)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -3019,16 +3015,16 @@
       </c>
       <c r="N3" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Kalau 3 dari 5 ini ada di CD kamu, buang. Sekarang." | Teks: 5 TANDA HARUS DIBUANG
-[3-28s] 1. Karet melar. 2. Kain menipis/nerawang. 3. Warna kusam permanen. 4. Bau nggak hilang walau dicuci. 5. Umur lebih dari setahun. (tiap poin 4-5 detik + angka besar)
-[28-33s] "Kena berapa poin? Komen di bawah."</t>
+          <t>[0-2s] "CD kamu harus dibuang kalau ada tanda ini."
+[2-12s] Cepat: "1 karet melar, 2 kain nerawang, 3 warna kusam, 4 bau nempel, 5 umur &gt;1 tahun."
+[12-15s] "Kena berapa? Komen."</t>
         </is>
       </c>
       <c r="O3" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook host to-camera.
-S2-S6 lima insert b-roll CD lama (blur) + angka overlay tiap tanda.
-S7 host CTA + gesture komen.</t>
+          <t>S1 [0-2s] Hook host.
+S2 [2-12s] 5 insert kilat CD lama (blur) + angka.
+S3 [12-15s] CTA komen.</t>
         </is>
       </c>
       <c r="P3" s="48" t="inlineStr">
@@ -3063,7 +3059,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Demo side-by-side</t>
+          <t>Demo side-by-side (≤15 dtk)</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -3099,19 +3095,16 @@
       </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "CD 100 ribu vs 10 ribu. Kita tarik sampai salah satu nyerah."
-[3-20s] "Dua-duanya ditarik dengan beban sama." (tarik pelan, makro serat)
-[20-30s] "Yang murah melar dan nggak balik. Yang ini balik lagi." (tunjuk recovery)
-[30-35s] "Kualitas kerasa dari tarikan pertama. Cek keranjang kuning."</t>
+          <t>[0-2s] "CD 100 ribu vs 10 ribu. Tarik sampai nyerah."
+[2-11s] (tarik dua-duanya) "Yang murah melar, yang ini balik lagi."
+[11-15s] "Keranjang kuning."</t>
         </is>
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook dua produk di tangan.
-S2 [3-20s] Wide dua tangan menarik bersamaan.
-S3 makro serat saat ditarik.
-S4 [20-30s] Side-by-side hasil recovery.
-S5 endcard CTA.</t>
+          <t>S1 [0-2s] Dua produk di tangan.
+S2 [2-11s] Tarik bareng + makro recovery.
+S3 [11-15s] Endcard CTA.</t>
         </is>
       </c>
       <c r="P4" s="48" t="inlineStr">
@@ -3146,7 +3139,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Talking head + ilustrasi</t>
+          <t>Talking head + ilustrasi (≤15 dtk)</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -3182,18 +3175,16 @@
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Area intim gampang gatal &amp; lembab? Bukan karena jorok."
-[3-12s] "Penyebabnya: bahan nggak breathable, lembab kejebak, gesekan jahitan."
-[12-28s] "Solusinya bukan bedak. Tapi pilih bahan yang bisa 'napas' dan jahitan yang halus." (tunjuk sampel bahan)
-[28-33s] "Share ke temanmu yang sering ngeluh."</t>
+          <t>[0-2s] "Area intim gatal? Bukan karena jorok."
+[2-12s] "Penyebabnya bahan nggak breathable + jahitan kasar. Solusinya bahan yang bisa napas."
+[12-15s] "Share ke temanmu."</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Host to-cam, ekspresi serius.
-S2 [3-12s] Grafis sederhana penyebab + b-roll kulit/kain (aman).
-S3 [12-28s] Insert sampel bahan breathable vs tidak.
-S4 CTA share.</t>
+          <t>S1 [0-2s] Host serius.
+S2 [2-12s] Insert sampel bahan breathable vs tidak.
+S3 [12-15s] CTA share.</t>
         </is>
       </c>
       <c r="P5" s="48" t="inlineStr">
@@ -3228,7 +3219,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Talking head listicle</t>
+          <t>Talking head listicle (≤15 dtk)</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -3264,18 +3255,16 @@
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Bukan jam. Bukan sepatu. Hal pertama yang bikin cowok keliatan mahal itu ini."
-[3-22s] "Tiga hal yang orang lain nggak lihat: wangi, kuku rapi, dan dalaman berkualitas."
-[22-30s] "Kemewahan yang kamu rasakan sendiri." (flat lay produk)
-[30-35s] "Mulai dari yang paling dalam. Link di bio."</t>
+          <t>[0-2s] "Bukan jam, bukan sepatu."
+[2-12s] "Yang bikin cowok keliatan mahal: wangi, kuku rapi, dalaman berkualitas."
+[12-15s] "Mulai dari dalam. Link di bio."</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Host to-cam berpakaian rapi.
-S2 [3-22s] 3 b-roll: parfum, gunting kuku, laci produk.
-S3 flat lay produk elegan.
-S4 endcard.</t>
+          <t>S1 [0-2s] Host rapi.
+S2 [2-12s] 3 b-roll kilat + flat lay produk.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P6" s="48" t="inlineStr">
@@ -3310,7 +3299,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Demo close-up satisfying</t>
+          <t>Demo close-up satisfying (≤15 dtk)</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -3346,18 +3335,16 @@
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Tuang air ke dua kain ini. Lihat mana yang 'minum' duluan."
-[3-18s] (slow-mo) air di kain murah menggenang; di kain Toni Black langsung menyerap.
-[18-26s] "Ini yang namanya moisture-wicking. Kering = kulit sehat."
-[26-31s] "Kulitmu tahu bedanya. Keranjang kuning."</t>
+          <t>[0-2s] "Tuang air ke dua kain ini."
+[2-11s] (slow-mo) "Yang murah menggenang. Yang ini langsung menyerap."
+[11-15s] "Kering = sehat. Keranjang kuning."</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook dua potong kain berlabel.
-S2 [3-18s] Makro slow-mo tetes air di dua kain.
-S3 [18-26s] Split-screen hasil serap.
-S4 endcard CTA.</t>
+          <t>S1 [0-2s] Dua kain berlabel.
+S2 [2-11s] Makro tetes air.
+S3 [11-15s] Split hasil + CTA.</t>
         </is>
       </c>
       <c r="P7" s="48" t="inlineStr">
@@ -3392,7 +3379,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>POV cinematic</t>
+          <t>POV cinematic (≤15 dtk)</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -3428,17 +3415,16 @@
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] VO: "Hal paling mahal yang dia pakai hari ini... nggak keliatan." | Teks sama.
-[3-22s] (sinematik, tanpa dialog) rutinitas pagi: kopi, skincare, kancing kemeja, buka laci berisi CD tersusun rapi (produk dilipat, tidak dipakai di kamera).
-[22-28s] Teks: UPGRADE DIMULAI DARI DALAM. | "Link di bio."</t>
+          <t>[0-2s] Teks: "Hal paling mahal yang dia pakai... nggak keliatan."
+[2-12s] (sinematik, tanpa dialog) kopi, skincare, kemeja, laci CD rapi.
+[12-15s] Teks: "Upgrade dari dalam."</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] CU wajah/tangan + teks hook.
-S2 [3-22s] Montase 4-5 shot cinematic pagi, gerak kamera halus.
-S3 CU laci produk rapi.
-S4 endcard teks.</t>
+          <t>S1 [0-2s] CU + teks hook.
+S2 [2-12s] 4 shot cinematic kilat.
+S3 [12-15s] CU laci + endcard.</t>
         </is>
       </c>
       <c r="P8" s="48" t="inlineStr">
@@ -3473,7 +3459,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Perbandingan bahan</t>
+          <t>Perbandingan bahan (≤15 dtk)</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -3509,17 +3495,16 @@
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Bahan CD kamu menentukan kesehatan kulitmu. Serius."
-[3-25s] Pegang 3 sampel: poliester murah (panas), katun biasa (nyerap tapi lama kering), micromodal premium (lembut + breathable). Jelaskan beda serat &amp; sirkulasi udara.
-[25-30s] "Save sebelum beli CD lagi."</t>
+          <t>[0-2s] "Bahan CD nentuin kesehatan kulitmu."
+[2-12s] (pegang 3 kain) "Poliester panas, katun lama kering, modal breathable + lembut."
+[12-15s] "Save sebelum beli."</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Host pegang 3 sampel.
-S2 [3-25s] Insert makro tiap kain + label nama bahan.
-S3 demo remas/tiup untuk breathability.
-S4 CTA save.</t>
+          <t>S1 [0-2s] 3 sampel di tangan.
+S2 [2-12s] Makro tiap kain + label.
+S3 [12-15s] CTA save.</t>
         </is>
       </c>
       <c r="P9" s="48" t="inlineStr">
@@ -3554,7 +3539,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Breakdown komponen</t>
+          <t>Breakdown komponen (≤15 dtk)</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -3590,17 +3575,16 @@
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Ini alasan kenapa 1 pcs harganya 100 ribu. Kita bedah."
-[3-45s] Bedah per bagian: gramasi bahan (timbang), jahitan flatlock (makro), waistband tenun (tarik), karet premium. Bandingkan diam-diam dengan CD murah yang juga dibedah.
-[45-55s] "Sekarang kamu tahu bayar untuk apa. Link di bio."</t>
+          <t>[0-2s] "Kenapa 1 pcs 100 ribu? Kita bedah."
+[2-12s] (potong cepat) "Gramasi tebal, jahitan flatlock, waistband tenun, karet premium."
+[12-15s] "Bayar untuk ini. Link di bio."</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook produk utuh + gunting.
-S2-S5 empat insert makro tiap komponen (bahan, jahitan, waistband, karet).
-S6 side-by-side vs CD murah terbedah.
-S7 endcard.</t>
+          <t>S1 [0-2s] Produk + gunting.
+S2 [2-12s] 4 makro komponen kilat.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P10" s="48" t="inlineStr">
@@ -3635,7 +3619,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>BTS QC</t>
+          <t>BTS QC (≤15 dtk)</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -3671,17 +3655,16 @@
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Yang nggak lolos QC, nggak kami diskon. Kami gunting."
-[3-25s] Proses QC: cek jahitan, tarik karet, terawang kain → temukan cacat → gunting produk gagal di depan kamera.
-[25-32s] "Ini standar yang kamu bayar. Follow untuk BTS lain."</t>
+          <t>[0-2s] "Yang gagal QC, kami gunting. Bukan didiskon."
+[2-12s] Cek jahitan/karet -&gt; temukan cacat -&gt; gunting.
+[12-15s] "Standar yang kamu bayar. Follow."</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] CU tangan pegang produk + gunting.
-S2 [3-25s] Beberapa insert proses cek QC di meja.
-S3 momen gunting (satisfying).
-S4 endcard.</t>
+          <t>S1 [0-2s] Tangan + gunting.
+S2 [2-12s] Cek kilat + momen gunting.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P11" s="48" t="inlineStr">
@@ -3716,7 +3699,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Talking head</t>
+          <t>Talking head (≤15 dtk)</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -3752,16 +3735,16 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Kamu pakai CD yang sama lebih dari setahun? Dengerin dulu."
-[3-20s] "Menurut dermatolog, CD idealnya dirotasi dan diganti total tiap 6-12 bulan. Kain lama menyimpan bakteri walau sudah dicuci."
-[20-27s] "Cek laci kamu malam ini."</t>
+          <t>[0-2s] "Pakai CD sama lebih dari setahun?"
+[2-12s] "Menurut dermatolog, ganti tiap 6-12 bulan. Kain lama simpan bakteri walau dicuci."
+[12-15s] "Cek lacimu malam ini."</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Host to-cam.
-S2 [3-20s] Text overlay angka '6-12 bulan' + b-roll laci CD.
-S3 CTA.</t>
+          <t>S1 [0-2s] Host.
+S2 [2-12s] Teks '6-12 bulan' + b-roll laci.
+S3 [12-15s] CTA.</t>
         </is>
       </c>
       <c r="P12" s="48" t="inlineStr">
@@ -3796,7 +3779,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Gift angle (audiens perempuan)</t>
+          <t>Gift angle (audiens perempuan) (≤15 dtk)</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -3832,17 +3815,16 @@
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Kado buat cowok itu gampang. Yang susah: kado yang dia PAKAI."
-[3-22s] "Parfum? Numpuk. Dompet? Udah punya. Tapi celana dalam premium — dipakai TIAP hari." (tunjuk gift box)
-[22-30s] Reaksi unboxing pasangan. "Tag pasanganmu. Gift box di keranjang kuning."</t>
+          <t>[0-2s] "Kado cowok yang susah: yang dia PAKAI."
+[2-12s] "Parfum numpuk, dompet udah punya. Tapi CD premium dipakai tiap hari." (gift box)
+[12-15s] "Tag pasanganmu."</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Talent perempuan to-cam pegang gift box.
-S2 [3-22s] B-roll kado 'gagal' vs gift box Toni Black.
-S3 [22-30s] Reaksi unboxing.
-S4 endcard CTA tag.</t>
+          <t>S1 [0-2s] Talent perempuan + gift box.
+S2 [2-12s] Kado gagal vs gift box.
+S3 [12-15s] CTA tag.</t>
         </is>
       </c>
       <c r="P13" s="48" t="inlineStr">
@@ -3877,7 +3859,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>ASMR unboxing</t>
+          <t>ASMR unboxing (≤15 dtk)</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -3913,16 +3895,17 @@
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>(Tanpa dialog — full ASMR) Teks awal: "Kado terbaik itu yang dipakai tiap hari."
-Urutan suara: buka sleeve box → tissue paper → angkat produk terlipat → kartu ucapan → tutup box.
-Teks akhir: "Kirim ke dia yang perlu upgrade."</t>
+          <t>(tanpa dialog, ASMR)
+[0-2s] Teks: "Kado yang dipakai tiap hari."
+[2-13s] suara buka box -&gt; tissue -&gt; produk -&gt; kartu.
+[13-15s] Teks: "Kirim ke dia."</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-4s] CU tangan buka box + teks.
-S2-S4 makro tiap tahap unboxing, suara asli dominan.
-S5 produk final di frame + teks CTA.</t>
+          <t>S1 [0-2s] CU buka box + teks.
+S2 [2-13s] Makro tahap unboxing.
+S3 [13-15s] Produk + teks.</t>
         </is>
       </c>
       <c r="P14" s="48" t="inlineStr">
@@ -3957,7 +3940,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>UGC/testimoni</t>
+          <t>UGC/testimoni (≤15 dtk)</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -3993,16 +3976,16 @@
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Aku beliin suamiku celana dalam 100 ribu. Reaksinya di luar dugaan."
-[3-25s] "Awalnya dia protes 'kemahalan'. Seminggu kemudian... dia minta dibeliin lagi." (screenshot chat asli, dengan izin)
-[25-30s] "Coba dulu 1 pcs. Keranjang kuning."</t>
+          <t>[0-2s] "Aku beliin suamiku CD 100 ribu."
+[2-12s] "Awalnya protes kemahalan. Seminggu kemudian minta dibeliin lagi." (screenshot chat)
+[12-15s] "Coba 1. Keranjang kuning."</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] UGC istri to-cam (natural, handheld).
-S2 [3-25s] Insert screenshot chat + b-roll produk.
-S3 CTA.</t>
+          <t>S1 [0-2s] UGC istri.
+S2 [2-12s] Screenshot chat + produk.
+S3 [12-15s] CTA.</t>
         </is>
       </c>
       <c r="P15" s="48" t="inlineStr">
@@ -4037,7 +4020,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Listicle cepat</t>
+          <t>Listicle cepat (≤15 dtk)</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -4073,16 +4056,16 @@
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Kesalahan nomor 2 dilakukan 90% pria Indonesia."
-[3-24s] 1. Beli karena murah per lusin. 2. Salah ukuran (ikut ukuran kaos). 3. Nggak lihat bahan. (tiap poin solusi singkat)
-[24-29s] "Kamu pernah yang mana? Komen."</t>
+          <t>[0-2s] "Kesalahan nomor 2 dilakukan 90% pria."
+[2-12s] "1 beli karena murah per lusin, 2 salah ukuran, 3 nggak lihat bahan."
+[12-15s] "Kamu yang mana? Komen."</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook host to-cam.
-S2-S4 tiga insert ilustrasi tiap kesalahan + angka.
-S5 CTA komen.</t>
+          <t>S1 [0-2s] Hook host.
+S2 [2-12s] 3 insert kilat.
+S3 [12-15s] CTA.</t>
         </is>
       </c>
       <c r="P16" s="48" t="inlineStr">
@@ -4117,7 +4100,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Demo uap</t>
+          <t>Demo uap (≤15 dtk)</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -4153,17 +4136,16 @@
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Kalau uap aja nggak bisa lewat, gimana kulitmu bisa napas?"
-[3-20s] Uap/hairdryer di balik dua kain: kain murah menahan uap; Toni Black tembus. "Ini bedanya breathable."
-[20-26s] "Kulit juga butuh napas. Link di bio."</t>
+          <t>[0-2s] "Uap aja nggak lewat, gimana kulitmu napas?"
+[2-12s] (uap di balik dua kain) "Yang murah nahan, yang ini tembus."
+[12-15s] "Link di bio."</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook dua kain di ring/frame.
-S2 [3-20s] Uap dari bawah, kamera samping, lihat tembus/tidak.
-S3 close-up perbandingan.
-S4 endcard.</t>
+          <t>S1 [0-2s] Dua kain di frame.
+S2 [2-12s] Uap dari bawah, lihat tembus.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P17" s="48" t="inlineStr">
@@ -4198,7 +4180,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Talking head + b-roll</t>
+          <t>Talking head + b-roll (≤15 dtk)</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
@@ -4234,16 +4216,16 @@
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Umur 30 ke atas, upgrade dulu barang yang kamu pakai TIAP HARI."
-[3-24s] "Konsep cost-per-wear: barang harian premium lebih masuk akal daripada barang pamer yang jarang dipakai. Kasur, sepatu harian... dan celana dalam."
-[24-30s] "Hitung cost-per-wear-mu. Link di bio."</t>
+          <t>[0-2s] "Umur 30+, upgrade yang kamu pakai TIAP hari dulu."
+[2-12s] "Cost-per-wear: barang harian premium lebih masuk akal dari barang pamer."
+[12-15s] "Link di bio."</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Host to-cam.
-S2 [3-24s] B-roll lifestyle + grafis hitung cost-per-wear.
-S3 endcard.</t>
+          <t>S1 [0-2s] Host.
+S2 [2-12s] B-roll + grafik cost-per-wear.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P18" s="48" t="inlineStr">
@@ -4278,7 +4260,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Mitos vs fakta</t>
+          <t>Mitos vs fakta (≤15 dtk)</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -4314,16 +4296,16 @@
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Katanya CD ketat itu bahaya. Mitos atau fakta?"
-[3-22s] "Yang penting bukan ketat atau longgar — tapi bahan breathable dan ukuran yang pas. Ini cara cek ukuranmu." (tunjuk size chart)
-[22-28s] "Save untuk referensi ukuran."</t>
+          <t>[0-2s] "CD ketat itu bahaya? Mitos atau fakta?"
+[2-12s] "Yang penting bukan ketat/longgar, tapi bahan breathable + ukuran pas."
+[12-15s] "Save referensi ukuran."</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook host, teks MITOS / FAKTA.
-S2 [3-22s] Insert size chart + demo ukur.
-S3 CTA save.</t>
+          <t>S1 [0-2s] Host + teks MITOS/FAKTA.
+S2 [2-12s] Size chart.
+S3 [12-15s] CTA save.</t>
         </is>
       </c>
       <c r="P19" s="48" t="inlineStr">
@@ -4358,7 +4340,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Reply-to-comment</t>
+          <t>Reply-to-comment (≤15 dtk)</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -4394,16 +4376,16 @@
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] (Reply to Comment) Screenshot komen: 'mending 10 pcs 100rb' → "Oke, kita hitung bareng."
-[3-25s] "CD murah rusak 2 bulan. Premium tahan 1,5-2 tahun. Bagi harga per hari... yang premium justru lebih murah." (grafik kalkulator on-screen)
-[25-30s] "Masih tim borongan? Komen di bawah."</t>
+          <t>[0-2s] (Reply komen 'mending 10 pcs 100rb') "Oke, kita hitung."
+[2-12s] "Murah rusak 2 bulan, premium 2 tahun. Per hari? Premium lebih murah."
+[12-15s] "Masih tim borongan?"</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Tempel screenshot komen (fitur Reply) + host.
-S2 [3-25s] Animasi hitung cost-per-wear.
-S3 host senyum, tanpa defensif.</t>
+          <t>S1 [0-2s] Screenshot komen + host.
+S2 [2-12s] Animasi hitung.
+S3 [12-15s] Host senyum.</t>
         </is>
       </c>
       <c r="P20" s="48" t="inlineStr">
@@ -4438,7 +4420,7 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Makro slow-mo</t>
+          <t>Makro slow-mo (≤15 dtk)</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -4474,17 +4456,16 @@
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Perbedaan 100 ribu itu ada di detail yang nggak pernah kamu perhatiin."
-[3-25s] (makro slow-mo) jahitan flatlock anti-gesek, tenunan waistband, label tanpa jahitan gatal. Side-by-side dengan jahitan CD murah yang kasar.
-[25-30s] "Detail itu mahal. Link di bio."</t>
+          <t>[0-2s] "Beda 100 ribu ada di detail ini."
+[2-12s] (makro) "Jahitan flatlock anti-gesek, waistband tenun, label tanpa gatal."
+[12-15s] "Detail itu mahal. Link di bio."</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook produk + teks.
-S2-S4 makro tiga detail (jahitan, waistband, label).
-S5 side-by-side vs murah.
-S6 endcard.</t>
+          <t>S1 [0-2s] Produk + teks.
+S2 [2-12s] 3 makro detail.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P21" s="48" t="inlineStr">
@@ -4519,7 +4500,7 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Packing video</t>
+          <t>Packing video (≤15 dtk)</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -4555,17 +4536,16 @@
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Business trip 3 hari, 1 tas kabin. Yang pertama masuk?"
-[3-22s] Packing rapi: kemeja digulung, pouch skincare, lalu pouch dalaman premium Toni Black masuk duluan.
-[22-28s] "Travel kit ada di keranjang kuning."</t>
+          <t>[0-2s] "Trip 3 hari, 1 tas kabin. Masuk pertama?"
+[2-12s] (packing cepat) kemeja gulung, pouch, CD premium masuk duluan.
+[12-15s] "Travel kit di keranjang kuning."</t>
         </is>
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook tas kabin terbuka.
-S2 [3-22s] Time-lapse/ritmis packing tiap item.
-S3 CU pouch produk.
-S4 endcard.</t>
+          <t>S1 [0-2s] Tas kabin.
+S2 [2-12s] Time-lapse packing.
+S3 [12-15s] CU pouch + CTA.</t>
         </is>
       </c>
       <c r="P22" s="48" t="inlineStr">
@@ -4600,7 +4580,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Tutorial singkat</t>
+          <t>Tutorial singkat (≤15 dtk)</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -4636,17 +4616,16 @@
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Barang 100 ribu dirawatnya beda. Ini caranya."
-[3-24s] 3 aturan: cuci lembut/tangan, jangan pengering panas, jemur terbalik tanpa matahari langsung. Bonus: cara melipat ala retail.
-[24-30s] "Save biar investasimu awet 2 tahun."</t>
+          <t>[0-2s] "Barang 100 ribu dirawatnya beda."
+[2-12s] "1 cuci lembut, 2 jangan pengering panas, 3 jemur terbalik."
+[12-15s] "Save biar awet 2 tahun."</t>
         </is>
       </c>
       <c r="O23" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Host pegang produk.
-S2-S4 tiga insert langkah perawatan.
-S5 demo lipat rapi.
-S6 CTA save.</t>
+          <t>S1 [0-2s] Host + produk.
+S2 [2-12s] 3 insert langkah.
+S3 [12-15s] CTA save.</t>
         </is>
       </c>
       <c r="P23" s="48" t="inlineStr">
@@ -4681,7 +4660,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Before/after + timelapse</t>
+          <t>Before/after + timelapse (≤15 dtk)</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -4717,17 +4696,16 @@
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "CD ini sudah dicuci 30 kali. Ini bentuknya sekarang."
-[3-22s] Bandingkan unit 30x cuci vs unit baru: warna, karet, bentuk. "Nyaris nggak ada beda." (timelapse dokumentasi cuci)
-[22-28s] "Ini yang kamu bayar. Keranjang kuning."</t>
+          <t>[0-2s] "CD ini udah dicuci 30 kali."
+[2-12s] (side-by-side lama vs baru) "Warna, karet, bentuk - nyaris sama."
+[12-15s] "Ini yang kamu bayar."</t>
         </is>
       </c>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook dua unit di tangan.
-S2 [3-22s] Timelapse cuci + side-by-side.
-S3 CU karet &amp; warna.
-S4 endcard.</t>
+          <t>S1 [0-2s] Dua unit di tangan.
+S2 [2-12s] Side-by-side + CU karet.
+S3 [12-15s] CTA.</t>
         </is>
       </c>
       <c r="P24" s="48" t="inlineStr">
@@ -4762,7 +4740,7 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Kompilasi review</t>
+          <t>Kompilasi review (≤15 dtk)</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -4798,16 +4776,16 @@
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Kata mereka yang sudah pindah ke Toni Black:"
-[3-24s] Kompilasi 3 screenshot review bintang 5 + voice over highlight ('lembut', 'adem', 'nggak balik lagi ke yang murah').
-[24-30s] "Buktikan sendiri. Keranjang kuning."</t>
+          <t>[0-2s] "Kata yang udah pindah ke Toni Black:"
+[2-12s] 3 review bintang 5 ('lembut', 'adem', 'nggak balik ke murah').
+[12-15s] "Buktikan sendiri."</t>
         </is>
       </c>
       <c r="O25" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook teks + b-roll produk.
-S2-S4 tiga kartu review animasi masuk.
-S5 endcard CTA.</t>
+          <t>S1 [0-2s] Hook + produk.
+S2 [2-12s] 3 kartu review animasi.
+S3 [12-15s] Endcard CTA.</t>
         </is>
       </c>
       <c r="P25" s="48" t="inlineStr">
@@ -4842,7 +4820,7 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>Listicle visual</t>
+          <t>Listicle visual (≤15 dtk)</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -4878,17 +4856,16 @@
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Isi tas gym pria yang rapi. Nomor 4 sering dilupakan."
-[3-24s] Sepatu, handuk, skincare mini, lalu CD ganti Toni Black (poin edukasi: keringat = lembab, wajib bawa ganti).
-[24-30s] "Jangan skip nomor 4. Link di bio."</t>
+          <t>[0-2s] "Isi tas gym pria rapi. Nomor 4 sering lupa."
+[2-12s] sepatu, handuk, skincare, CD ganti (keringat=lembab, wajib ganti).
+[12-15s] "Jangan skip nomor 4."</t>
         </is>
       </c>
       <c r="O26" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook tas gym + teks.
-S2 [3-24s] Keluarkan item satu-satu + angka overlay.
-S3 CU produk 'nomor 4'.
-S4 endcard.</t>
+          <t>S1 [0-2s] Tas gym.
+S2 [2-12s] Keluarkan item + angka.
+S3 [12-15s] CU produk + CTA.</t>
         </is>
       </c>
       <c r="P26" s="48" t="inlineStr">
@@ -4923,7 +4900,7 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>Edukasi + soft sell</t>
+          <t>Edukasi + soft sell (≤15 dtk)</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -4959,16 +4936,16 @@
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Punya CD banyak itu bukan boros. Ini hitungannya."
-[3-22s] "Sistem rotasi 7+ pcs: tiap kain 'istirahat' setelah dipakai jadi lebih awet, dan kamu selalu punya yang kering." (tunjuk laci tersusun)
-[22-30s] "Lengkapi rotasimu. Bundle hemat di keranjang kuning."</t>
+          <t>[0-2s] "Punya CD banyak bukan boros."
+[2-12s] "Rotasi 7+: kain istirahat jadi awet, selalu ada yang kering."
+[12-15s] "Lengkapi rotasimu. Bundle di keranjang kuning."</t>
         </is>
       </c>
       <c r="O27" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook laci penuh CD rapi.
-S2 [3-22s] Grafis rotasi 7 hari + b-roll.
-S3 CTA bundle.</t>
+          <t>S1 [0-2s] Laci penuh rapi.
+S2 [2-12s] Grafis rotasi 7 hari.
+S3 [12-15s] CTA bundle.</t>
         </is>
       </c>
       <c r="P27" s="48" t="inlineStr">
@@ -5003,7 +4980,7 @@
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>BTS produksi</t>
+          <t>BTS produksi (≤15 dtk)</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -5039,16 +5016,16 @@
       </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "100 ribu itu bukan harga kain. Ini prosesnya."
-[3-30s] Perjalanan produk: pilih kain → cutting → jahit → QC → packing. 5-6 detik per tahap + text overlay nama tahap.
-[30-36s] "Sekarang kamu tahu prosesnya. Follow untuk BTS lain."</t>
+          <t>[0-2s] "100 ribu bukan harga kain. Ini prosesnya."
+[2-12s] (kilat) pilih kain -&gt; cutting -&gt; jahit -&gt; QC -&gt; packing.
+[12-15s] "Follow untuk BTS lain."</t>
         </is>
       </c>
       <c r="O28" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook gulungan kain/workshop.
-S2-S6 lima shot tiap tahap produksi.
-S7 endcard.</t>
+          <t>S1 [0-2s] Gulungan kain.
+S2 [2-12s] 5 shot tahap produksi kilat.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P28" s="48" t="inlineStr">
@@ -5083,7 +5060,7 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>Light education</t>
+          <t>Light education (≤15 dtk)</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -5119,16 +5096,16 @@
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Ada alasannya kenapa CD terbaik di dunia kebanyakan warna gelap."
-[3-20s] "Noda &amp; kusam nggak keliatan, terlihat baru lebih lama, dan netral di balik semua outfit." (tunjuk lini warna)
-[20-26s] "Tim hitam atau tim navy? Komen."</t>
+          <t>[0-2s] "Kenapa CD terbaik kebanyakan warna gelap?"
+[2-12s] "Noda &amp; kusam nggak keliatan, terlihat baru lebih lama, netral di semua outfit."
+[12-15s] "Tim hitam atau navy? Komen."</t>
         </is>
       </c>
       <c r="O29" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook host + flat lay warna gelap.
-S2 [3-20s] B-roll produk beberapa warna.
-S3 CTA komen.</t>
+          <t>S1 [0-2s] Flat lay gelap.
+S2 [2-12s] B-roll warna.
+S3 [12-15s] CTA komen.</t>
         </is>
       </c>
       <c r="P29" s="48" t="inlineStr">
@@ -5163,7 +5140,7 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>Demo timbangan</t>
+          <t>Demo timbangan (≤15 dtk)</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
@@ -5199,17 +5176,16 @@
       </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Kain CD itu ada 'kelasnya'. Kita timbang biar jujur."
-[3-22s] Timbang kain CD murah vs Toni Black (ukuran sama). "Gramasi lebih tinggi = kain lebih padat &amp; tahan lama. Namanya GSM."
-[22-28s] "Sekarang kamu ngerti GSM. Link di bio."</t>
+          <t>[0-2s] "Kain CD ada kelasnya. Kita timbang."
+[2-12s] (timbang murah vs Toni Black) "Gramasi tinggi = padat &amp; awet. Namanya GSM."
+[12-15s] "Link di bio."</t>
         </is>
       </c>
       <c r="O30" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Hook timbangan digital + kain.
-S2 [3-22s] Timbang dua kain, CU angka.
-S3 grafik GSM.
-S4 endcard.</t>
+          <t>S1 [0-2s] Timbangan + kain.
+S2 [2-12s] Timbang dua kain + CU angka.
+S3 [12-15s] Endcard.</t>
         </is>
       </c>
       <c r="P30" s="48" t="inlineStr">
@@ -5244,7 +5220,7 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>Short promo momen payday</t>
+          <t>Short promo momen payday (≤15 dtk)</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -5280,16 +5256,16 @@
       </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
-          <t>[0-3s] "Gajian sudah masuk. Upgrade dulu barang yang kamu pakai TIAP HARI."
-[3-18s] Recap cuplikan demo terbaik bulan ini (stretch test, tes serap air) + tunjukkan bundle gift box edisi gajian.
-[18-25s] "Checkout gift box edisi gajian sekarang di keranjang kuning."</t>
+          <t>[0-2s] "Gajian masuk. Upgrade yang kamu pakai tiap hari."
+[2-12s] cuplikan demo terbaik + gift box edisi gajian.
+[12-15s] "Checkout gift box di keranjang kuning." (TANPA live)</t>
         </is>
       </c>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>S1 [0-3s] Host energik + teks GAJIAN.
-S2 [3-18s] Montase cuplikan demo + gift box.
-S3 [18-25s] Endcard produk + CTA keranjang kuning.</t>
+          <t>S1 [0-2s] Host + teks GAJIAN.
+S2 [2-12s] Montase demo + gift box.
+S3 [12-15s] Endcard CTA.</t>
         </is>
       </c>
       <c r="P31" s="48" t="inlineStr">

</xml_diff>